<commit_message>
[200~Update production_system_intake.xlsx with new version. I seem to have resolved an issue in an ingesttion test by chnaging the resources to more of a task resource matrix. This is not a great data model because there are a finite structure to the resources, but for an excel intake I think this works for now, till I can think of a better way.
</commit_message>
<xml_diff>
--- a/production_system_intake.xlsx
+++ b/production_system_intake.xlsx
@@ -5,25 +5,28 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Classes\2025_01_Spring\ASU\Computation\Week04\New folder\Intake\V01\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Classes\2025_01_Spring\ASU\Computation\Week04\New folder\Intake\V02\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAFCE1C4-6CAE-4637-8C0F-A46B20DD3410}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{817DD534-40BA-4B95-954C-C375E24C2EC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="2130" windowWidth="29040" windowHeight="15840" tabRatio="1000" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="2130" windowWidth="29040" windowHeight="15840" tabRatio="857" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="LocationTbl" sheetId="4" r:id="rId1"/>
-    <sheet name="ProcessorTbl" sheetId="5" r:id="rId2"/>
-    <sheet name="ProcessorTypeTbl" sheetId="3" r:id="rId3"/>
+    <sheet name="ProcessorTypeTbl" sheetId="3" r:id="rId1"/>
+    <sheet name="LocationTbl" sheetId="4" r:id="rId2"/>
+    <sheet name="ProcessorTbl" sheetId="5" r:id="rId3"/>
     <sheet name="TaskTbl" sheetId="1" r:id="rId4"/>
+    <sheet name="ResourceTbl" sheetId="2" r:id="rId5"/>
+    <sheet name="TaskResourcesTbl" sheetId="18" r:id="rId6"/>
+    <sheet name="StationTbl" sheetId="6" r:id="rId7"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="95">
   <si>
     <t>TaskIndex</t>
   </si>
@@ -76,6 +79,27 @@
     <t>ComponentsGenerated</t>
   </si>
   <si>
+    <t>ResourceIndex</t>
+  </si>
+  <si>
+    <t>ResourceName</t>
+  </si>
+  <si>
+    <t>ResourceType</t>
+  </si>
+  <si>
+    <t>TotalResourceUnitsAvailable</t>
+  </si>
+  <si>
+    <t>DownProbabilityPerUnit</t>
+  </si>
+  <si>
+    <t>DownReplacementDelay</t>
+  </si>
+  <si>
+    <t>Units</t>
+  </si>
+  <si>
     <t>ProcessorTypeIndex</t>
   </si>
   <si>
@@ -112,7 +136,181 @@
     <t>ProcessingUnits</t>
   </si>
   <si>
+    <t>StationIndex</t>
+  </si>
+  <si>
+    <t>StationID</t>
+  </si>
+  <si>
+    <t>StationDesc</t>
+  </si>
+  <si>
+    <t>StationType</t>
+  </si>
+  <si>
+    <t>StationPriorityMethod</t>
+  </si>
+  <si>
+    <t>StationCapacity</t>
+  </si>
+  <si>
+    <t>DownProabilityPerUnit</t>
+  </si>
+  <si>
     <t>TasksDesc</t>
+  </si>
+  <si>
+    <t>NResource01</t>
+  </si>
+  <si>
+    <t>NResource02</t>
+  </si>
+  <si>
+    <t>NResource03</t>
+  </si>
+  <si>
+    <t>NResource04</t>
+  </si>
+  <si>
+    <t>NResource05</t>
+  </si>
+  <si>
+    <t>NResource06</t>
+  </si>
+  <si>
+    <t>NResource07</t>
+  </si>
+  <si>
+    <t>NResource08</t>
+  </si>
+  <si>
+    <t>NResource09</t>
+  </si>
+  <si>
+    <t>NResource10</t>
+  </si>
+  <si>
+    <t>NResource11</t>
+  </si>
+  <si>
+    <t>NResource12</t>
+  </si>
+  <si>
+    <t>NResource13</t>
+  </si>
+  <si>
+    <t>NResource14</t>
+  </si>
+  <si>
+    <t>NResource15</t>
+  </si>
+  <si>
+    <t>NResource16</t>
+  </si>
+  <si>
+    <t>NResource17</t>
+  </si>
+  <si>
+    <t>NResource18</t>
+  </si>
+  <si>
+    <t>NResource19</t>
+  </si>
+  <si>
+    <t>NResource20</t>
+  </si>
+  <si>
+    <t>NResource21</t>
+  </si>
+  <si>
+    <t>NResource22</t>
+  </si>
+  <si>
+    <t>NResource23</t>
+  </si>
+  <si>
+    <t>NResource24</t>
+  </si>
+  <si>
+    <t>NResource25</t>
+  </si>
+  <si>
+    <t>NResource26</t>
+  </si>
+  <si>
+    <t>NResource27</t>
+  </si>
+  <si>
+    <t>NResource28</t>
+  </si>
+  <si>
+    <t>NResource29</t>
+  </si>
+  <si>
+    <t>NResource30</t>
+  </si>
+  <si>
+    <t>NResource31</t>
+  </si>
+  <si>
+    <t>NResource32</t>
+  </si>
+  <si>
+    <t>NResource33</t>
+  </si>
+  <si>
+    <t>NResource34</t>
+  </si>
+  <si>
+    <t>NResource35</t>
+  </si>
+  <si>
+    <t>NResource36</t>
+  </si>
+  <si>
+    <t>NResource37</t>
+  </si>
+  <si>
+    <t>NResource38</t>
+  </si>
+  <si>
+    <t>NResource39</t>
+  </si>
+  <si>
+    <t>NResource40</t>
+  </si>
+  <si>
+    <t>NResource41</t>
+  </si>
+  <si>
+    <t>NResource42</t>
+  </si>
+  <si>
+    <t>NResource43</t>
+  </si>
+  <si>
+    <t>NResource44</t>
+  </si>
+  <si>
+    <t>NResource45</t>
+  </si>
+  <si>
+    <t>NResource46</t>
+  </si>
+  <si>
+    <t>NResource47</t>
+  </si>
+  <si>
+    <t>NResource48</t>
+  </si>
+  <si>
+    <t>NResource49</t>
+  </si>
+  <si>
+    <t>NResource50</t>
+  </si>
+  <si>
+    <t>ResourceID</t>
   </si>
 </sst>
 </file>
@@ -484,6 +682,32 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -496,16 +720,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -514,7 +738,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:M1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -545,64 +769,38 @@
         <v>4</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -640,7 +838,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -695,4 +893,294 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E098E04-19A8-4E79-81CD-069FB2C95590}">
+  <dimension ref="A1:BA29"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="53" width="12.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:53" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="AL1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="AN1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="AO1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="AP1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="AQ1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="AR1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="AS1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="AT1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="AU1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="AV1" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="AW1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="AX1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="AY1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="AZ1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="BA1" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="29" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C29" s="2"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:L1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update production_system_intake.xlsx with new version. Local testing seems to work well for my test ingestion of this intake form with the example. This adds intake for system components, producttypes, configurations, and arrival units and processing units. The idea is that as units arrive there the becomp componts and resources fr tasks at processors. I am still tryignt o resolf issues with have I do arrivals and delivery for intake.
</commit_message>
<xml_diff>
--- a/production_system_intake.xlsx
+++ b/production_system_intake.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Classes\2025_01_Spring\ASU\Computation\Week04\New folder\Intake\V02\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Classes\2025_01_Spring\ASU\Computation\Week04\New folder\Intake\V03\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{817DD534-40BA-4B95-954C-C375E24C2EC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B41F5B8-269F-4730-BB7A-100FC1DCD301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="2130" windowWidth="29040" windowHeight="15840" tabRatio="857" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="2130" windowWidth="29040" windowHeight="15840" tabRatio="857" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProcessorTypeTbl" sheetId="3" r:id="rId1"/>
@@ -20,13 +20,18 @@
     <sheet name="ResourceTbl" sheetId="2" r:id="rId5"/>
     <sheet name="TaskResourcesTbl" sheetId="18" r:id="rId6"/>
     <sheet name="StationTbl" sheetId="6" r:id="rId7"/>
+    <sheet name="ProductsTbl" sheetId="7" r:id="rId8"/>
+    <sheet name="ConfigTbl" sheetId="8" r:id="rId9"/>
+    <sheet name="ProcessUnitTbl" sheetId="9" r:id="rId10"/>
+    <sheet name="ArrivalUnitTbl" sheetId="10" r:id="rId11"/>
+    <sheet name="ComponentsTbl" sheetId="11" r:id="rId12"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="114">
   <si>
     <t>TaskIndex</t>
   </si>
@@ -155,6 +160,63 @@
   </si>
   <si>
     <t>DownProabilityPerUnit</t>
+  </si>
+  <si>
+    <t>ProductIndex</t>
+  </si>
+  <si>
+    <t>ProductID</t>
+  </si>
+  <si>
+    <t>ProductDesc</t>
+  </si>
+  <si>
+    <t>ConfigIndex</t>
+  </si>
+  <si>
+    <t>ConfigID</t>
+  </si>
+  <si>
+    <t>ConfigDesc</t>
+  </si>
+  <si>
+    <t>ProcessUnitIndex</t>
+  </si>
+  <si>
+    <t>ProcessUnitID</t>
+  </si>
+  <si>
+    <t>ProcessUnitDesc</t>
+  </si>
+  <si>
+    <t>ArrivalUnitIndex</t>
+  </si>
+  <si>
+    <t>ArrivalUnitID</t>
+  </si>
+  <si>
+    <t>ArrivalUnitDesc</t>
+  </si>
+  <si>
+    <t>ComponentIndex</t>
+  </si>
+  <si>
+    <t>ComponentID</t>
+  </si>
+  <si>
+    <t>ComponentDesc</t>
+  </si>
+  <si>
+    <t>UnitType</t>
+  </si>
+  <si>
+    <t>UnitIndex</t>
+  </si>
+  <si>
+    <t>UnitID</t>
+  </si>
+  <si>
+    <t>UnitDesc</t>
   </si>
   <si>
     <t>TasksDesc</t>
@@ -707,6 +769,171 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D1"/>
@@ -838,7 +1065,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -915,7 +1142,7 @@
         <v>17</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>94</v>
+        <v>113</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>18</v>
@@ -960,157 +1187,157 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>47</v>
+        <v>66</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>48</v>
+        <v>67</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>50</v>
+        <v>69</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>53</v>
+        <v>72</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>55</v>
+        <v>74</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>57</v>
+        <v>76</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>58</v>
+        <v>77</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>59</v>
+        <v>78</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>61</v>
+        <v>80</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>62</v>
+        <v>81</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>64</v>
+        <v>83</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>66</v>
+        <v>85</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>67</v>
+        <v>86</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>69</v>
+        <v>88</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>71</v>
+        <v>90</v>
       </c>
       <c r="AF1" s="1" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
       <c r="AH1" s="1" t="s">
-        <v>74</v>
+        <v>93</v>
       </c>
       <c r="AI1" s="1" t="s">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="AJ1" s="1" t="s">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="AK1" s="1" t="s">
-        <v>77</v>
+        <v>96</v>
       </c>
       <c r="AL1" s="1" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="AM1" s="1" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="AN1" s="1" t="s">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="AO1" s="1" t="s">
-        <v>81</v>
+        <v>100</v>
       </c>
       <c r="AP1" s="1" t="s">
-        <v>82</v>
+        <v>101</v>
       </c>
       <c r="AQ1" s="1" t="s">
-        <v>83</v>
+        <v>102</v>
       </c>
       <c r="AR1" s="1" t="s">
-        <v>84</v>
+        <v>103</v>
       </c>
       <c r="AS1" s="1" t="s">
-        <v>85</v>
+        <v>104</v>
       </c>
       <c r="AT1" s="1" t="s">
-        <v>86</v>
+        <v>105</v>
       </c>
       <c r="AU1" s="1" t="s">
-        <v>87</v>
+        <v>106</v>
       </c>
       <c r="AV1" s="1" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="AW1" s="1" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="AX1" s="1" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="AY1" s="1" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="AZ1" s="1" t="s">
-        <v>92</v>
+        <v>111</v>
       </c>
       <c r="BA1" s="1" t="s">
-        <v>93</v>
+        <v>112</v>
       </c>
     </row>
     <row r="29" spans="3:3" x14ac:dyDescent="0.25">
@@ -1183,4 +1410,68 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update production_system_intake.xlsx with new version. I decided to do a precidence matrix instad of a list for now. I will likely covert to a list later, but I am having some issue with ingestion att. I am working on personnel intake model elements and Ill have an example soon to follow.
</commit_message>
<xml_diff>
--- a/production_system_intake.xlsx
+++ b/production_system_intake.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Classes\2025_01_Spring\ASU\Computation\Week04\New folder\Intake\V03\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Classes\2025_01_Spring\ASU\Computation\Week04\New folder\Intake\V04\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B41F5B8-269F-4730-BB7A-100FC1DCD301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA4AEF3C-A0C9-4474-ADED-D4BD4162BD77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="2130" windowWidth="29040" windowHeight="15840" tabRatio="857" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="2130" windowWidth="29040" windowHeight="15840" tabRatio="857" firstSheet="5" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProcessorTypeTbl" sheetId="3" r:id="rId1"/>
@@ -20,18 +20,23 @@
     <sheet name="ResourceTbl" sheetId="2" r:id="rId5"/>
     <sheet name="TaskResourcesTbl" sheetId="18" r:id="rId6"/>
     <sheet name="StationTbl" sheetId="6" r:id="rId7"/>
-    <sheet name="ProductsTbl" sheetId="7" r:id="rId8"/>
-    <sheet name="ConfigTbl" sheetId="8" r:id="rId9"/>
-    <sheet name="ProcessUnitTbl" sheetId="9" r:id="rId10"/>
-    <sheet name="ArrivalUnitTbl" sheetId="10" r:id="rId11"/>
-    <sheet name="ComponentsTbl" sheetId="11" r:id="rId12"/>
+    <sheet name="ConfigTbl" sheetId="8" r:id="rId8"/>
+    <sheet name="ProcessUnitTbl" sheetId="9" r:id="rId9"/>
+    <sheet name="ArrivalUnitTbl" sheetId="10" r:id="rId10"/>
+    <sheet name="ComponentsTbl" sheetId="11" r:id="rId11"/>
+    <sheet name="ProductsTbl" sheetId="7" r:id="rId12"/>
+    <sheet name="Product01" sheetId="13" r:id="rId13"/>
+    <sheet name="ArrivalRatesTbl" sheetId="14" r:id="rId14"/>
+    <sheet name="ArrivalDatesTbl" sheetId="15" r:id="rId15"/>
+    <sheet name="DeliveryRatesTbl" sheetId="16" r:id="rId16"/>
+    <sheet name="DeliveryDatesTbl" sheetId="17" r:id="rId17"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="210">
   <si>
     <t>TaskIndex</t>
   </si>
@@ -84,6 +89,246 @@
     <t>ComponentsGenerated</t>
   </si>
   <si>
+    <t>task001</t>
+  </si>
+  <si>
+    <t>task002</t>
+  </si>
+  <si>
+    <t>task003</t>
+  </si>
+  <si>
+    <t>task004</t>
+  </si>
+  <si>
+    <t>task005</t>
+  </si>
+  <si>
+    <t>task006</t>
+  </si>
+  <si>
+    <t>task007</t>
+  </si>
+  <si>
+    <t>task008</t>
+  </si>
+  <si>
+    <t>task009</t>
+  </si>
+  <si>
+    <t>task010</t>
+  </si>
+  <si>
+    <t>task011</t>
+  </si>
+  <si>
+    <t>task012</t>
+  </si>
+  <si>
+    <t>task013</t>
+  </si>
+  <si>
+    <t>task014</t>
+  </si>
+  <si>
+    <t>task015</t>
+  </si>
+  <si>
+    <t>task016</t>
+  </si>
+  <si>
+    <t>task017</t>
+  </si>
+  <si>
+    <t>task018</t>
+  </si>
+  <si>
+    <t>task019</t>
+  </si>
+  <si>
+    <t>task020</t>
+  </si>
+  <si>
+    <t>task021</t>
+  </si>
+  <si>
+    <t>task022</t>
+  </si>
+  <si>
+    <t>task023</t>
+  </si>
+  <si>
+    <t>task024</t>
+  </si>
+  <si>
+    <t>task025</t>
+  </si>
+  <si>
+    <t>task026</t>
+  </si>
+  <si>
+    <t>task027</t>
+  </si>
+  <si>
+    <t>task028</t>
+  </si>
+  <si>
+    <t>task029</t>
+  </si>
+  <si>
+    <t>task030</t>
+  </si>
+  <si>
+    <t>task031</t>
+  </si>
+  <si>
+    <t>task032</t>
+  </si>
+  <si>
+    <t>task033</t>
+  </si>
+  <si>
+    <t>task034</t>
+  </si>
+  <si>
+    <t>task035</t>
+  </si>
+  <si>
+    <t>task036</t>
+  </si>
+  <si>
+    <t>task037</t>
+  </si>
+  <si>
+    <t>task038</t>
+  </si>
+  <si>
+    <t>task039</t>
+  </si>
+  <si>
+    <t>task040</t>
+  </si>
+  <si>
+    <t>task041</t>
+  </si>
+  <si>
+    <t>task042</t>
+  </si>
+  <si>
+    <t>task043</t>
+  </si>
+  <si>
+    <t>task044</t>
+  </si>
+  <si>
+    <t>task045</t>
+  </si>
+  <si>
+    <t>task046</t>
+  </si>
+  <si>
+    <t>task047</t>
+  </si>
+  <si>
+    <t>task048</t>
+  </si>
+  <si>
+    <t>task049</t>
+  </si>
+  <si>
+    <t>task050</t>
+  </si>
+  <si>
+    <t>task051</t>
+  </si>
+  <si>
+    <t>task052</t>
+  </si>
+  <si>
+    <t>task053</t>
+  </si>
+  <si>
+    <t>task054</t>
+  </si>
+  <si>
+    <t>task055</t>
+  </si>
+  <si>
+    <t>task056</t>
+  </si>
+  <si>
+    <t>task057</t>
+  </si>
+  <si>
+    <t>task058</t>
+  </si>
+  <si>
+    <t>task059</t>
+  </si>
+  <si>
+    <t>task060</t>
+  </si>
+  <si>
+    <t>task061</t>
+  </si>
+  <si>
+    <t>task062</t>
+  </si>
+  <si>
+    <t>task063</t>
+  </si>
+  <si>
+    <t>task064</t>
+  </si>
+  <si>
+    <t>task065</t>
+  </si>
+  <si>
+    <t>task066</t>
+  </si>
+  <si>
+    <t>task067</t>
+  </si>
+  <si>
+    <t>task068</t>
+  </si>
+  <si>
+    <t>task069</t>
+  </si>
+  <si>
+    <t>task070</t>
+  </si>
+  <si>
+    <t>task071</t>
+  </si>
+  <si>
+    <t>task072</t>
+  </si>
+  <si>
+    <t>task073</t>
+  </si>
+  <si>
+    <t>task074</t>
+  </si>
+  <si>
+    <t>task075</t>
+  </si>
+  <si>
+    <t>task076</t>
+  </si>
+  <si>
+    <t>task077</t>
+  </si>
+  <si>
+    <t>task078</t>
+  </si>
+  <si>
+    <t>task079</t>
+  </si>
+  <si>
+    <t>task080</t>
+  </si>
+  <si>
     <t>ResourceIndex</t>
   </si>
   <si>
@@ -372,14 +617,65 @@
     <t>NResource50</t>
   </si>
   <si>
+    <t>TaskPred</t>
+  </si>
+  <si>
     <t>ResourceID</t>
+  </si>
+  <si>
+    <t>ArrivalDatesIndex</t>
+  </si>
+  <si>
+    <t>ArrivalDatesID</t>
+  </si>
+  <si>
+    <t>ArrivalDatesDesc</t>
+  </si>
+  <si>
+    <t>ArrivalDate</t>
+  </si>
+  <si>
+    <t>ArrivalCount</t>
+  </si>
+  <si>
+    <t>ArrivalRatesIndex</t>
+  </si>
+  <si>
+    <t>ArrivalRatesID</t>
+  </si>
+  <si>
+    <t>ArrivalRatesDesc</t>
+  </si>
+  <si>
+    <t>ArrivalValue</t>
+  </si>
+  <si>
+    <t>ArrivalUnits</t>
+  </si>
+  <si>
+    <t>DeliveryRatesIndex</t>
+  </si>
+  <si>
+    <t>DeliveryRatesID</t>
+  </si>
+  <si>
+    <t>DeliveryRatesDesc</t>
+  </si>
+  <si>
+    <t>DeliveryRateDate</t>
+  </si>
+  <si>
+    <t>DeliveryCount</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -398,6 +694,13 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -435,13 +738,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -755,13 +1062,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>24</v>
+        <v>104</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>25</v>
+        <v>105</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>26</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -770,56 +1077,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:I1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -837,31 +1094,31 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>52</v>
+        <v>132</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>53</v>
+        <v>133</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>54</v>
+        <v>134</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>46</v>
+        <v>126</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>47</v>
+        <v>127</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>48</v>
+        <v>128</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>43</v>
+        <v>123</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>44</v>
+        <v>124</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>45</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -869,7 +1126,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:M1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -890,44 +1147,943 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
+  <dimension ref="A1:CC81"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="81" width="7.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:81" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="B1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" t="s">
+        <v>25</v>
+      </c>
+      <c r="K1" t="s">
+        <v>26</v>
+      </c>
+      <c r="L1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" t="s">
+        <v>28</v>
+      </c>
+      <c r="N1" t="s">
+        <v>29</v>
+      </c>
+      <c r="O1" t="s">
+        <v>30</v>
+      </c>
+      <c r="P1" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>32</v>
+      </c>
+      <c r="R1" t="s">
+        <v>33</v>
+      </c>
+      <c r="S1" t="s">
+        <v>34</v>
+      </c>
+      <c r="T1" t="s">
+        <v>35</v>
+      </c>
+      <c r="U1" t="s">
+        <v>36</v>
+      </c>
+      <c r="V1" t="s">
+        <v>37</v>
+      </c>
+      <c r="W1" t="s">
+        <v>38</v>
+      </c>
+      <c r="X1" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>40</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>47</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>50</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>51</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>52</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>53</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AN1" t="s">
         <v>55</v>
       </c>
+      <c r="AO1" t="s">
+        <v>56</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>57</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>58</v>
+      </c>
+      <c r="AR1" t="s">
+        <v>59</v>
+      </c>
+      <c r="AS1" t="s">
+        <v>60</v>
+      </c>
+      <c r="AT1" t="s">
+        <v>61</v>
+      </c>
+      <c r="AU1" t="s">
+        <v>62</v>
+      </c>
+      <c r="AV1" t="s">
+        <v>63</v>
+      </c>
+      <c r="AW1" t="s">
+        <v>64</v>
+      </c>
+      <c r="AX1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AY1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AZ1" t="s">
+        <v>67</v>
+      </c>
+      <c r="BA1" t="s">
+        <v>68</v>
+      </c>
+      <c r="BB1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BC1" t="s">
+        <v>70</v>
+      </c>
+      <c r="BD1" t="s">
+        <v>71</v>
+      </c>
+      <c r="BE1" t="s">
+        <v>72</v>
+      </c>
+      <c r="BF1" t="s">
+        <v>73</v>
+      </c>
+      <c r="BG1" t="s">
+        <v>74</v>
+      </c>
+      <c r="BH1" t="s">
+        <v>75</v>
+      </c>
+      <c r="BI1" t="s">
+        <v>76</v>
+      </c>
+      <c r="BJ1" t="s">
+        <v>77</v>
+      </c>
+      <c r="BK1" t="s">
+        <v>78</v>
+      </c>
+      <c r="BL1" t="s">
+        <v>79</v>
+      </c>
+      <c r="BM1" t="s">
+        <v>80</v>
+      </c>
+      <c r="BN1" t="s">
+        <v>81</v>
+      </c>
+      <c r="BO1" t="s">
+        <v>82</v>
+      </c>
+      <c r="BP1" t="s">
+        <v>83</v>
+      </c>
+      <c r="BQ1" t="s">
+        <v>84</v>
+      </c>
+      <c r="BR1" t="s">
+        <v>85</v>
+      </c>
+      <c r="BS1" t="s">
+        <v>86</v>
+      </c>
+      <c r="BT1" t="s">
+        <v>87</v>
+      </c>
+      <c r="BU1" t="s">
+        <v>88</v>
+      </c>
+      <c r="BV1" t="s">
+        <v>89</v>
+      </c>
+      <c r="BW1" t="s">
+        <v>90</v>
+      </c>
+      <c r="BX1" t="s">
+        <v>91</v>
+      </c>
+      <c r="BY1" t="s">
+        <v>92</v>
+      </c>
+      <c r="BZ1" t="s">
+        <v>93</v>
+      </c>
+      <c r="CA1" t="s">
+        <v>94</v>
+      </c>
+      <c r="CB1" t="s">
+        <v>95</v>
+      </c>
+      <c r="CC1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" spans="1:81" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:81" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:81" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:81" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:81" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:81" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:81" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:81" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:81" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:81" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:81" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:81" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:81" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:81" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:81" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>96</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
+  <dimension ref="A1:L1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>200</v>
+      </c>
       <c r="B1" s="1" t="s">
-        <v>56</v>
+        <v>201</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>57</v>
+        <v>202</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>58</v>
+        <v>203</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>198</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>59</v>
+        <v>199</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>60</v>
+        <v>132</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>61</v>
+        <v>133</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>46</v>
+        <v>134</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>47</v>
+        <v>123</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>48</v>
+        <v>124</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>45</v>
-      </c>
+        <v>125</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B2" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -947,16 +2103,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>107</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>108</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>29</v>
+        <v>109</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>30</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -996,34 +2152,34 @@
         <v>4</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>24</v>
+        <v>104</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>25</v>
+        <v>105</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>26</v>
+        <v>106</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>31</v>
+        <v>111</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>27</v>
+        <v>107</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>28</v>
+        <v>108</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>32</v>
+        <v>112</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>33</v>
+        <v>113</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>34</v>
+        <v>114</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>35</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -1065,7 +2221,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>62</v>
+        <v>142</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -1114,7 +2270,7 @@
       </c>
     </row>
     <row r="29" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C29" s="2"/>
+      <c r="C29" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1139,28 +2295,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>97</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>113</v>
+        <v>194</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>18</v>
+        <v>98</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>19</v>
+        <v>99</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>21</v>
+        <v>101</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>22</v>
+        <v>102</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>23</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -1187,161 +2343,161 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>62</v>
+        <v>142</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>63</v>
+        <v>143</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>64</v>
+        <v>144</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>65</v>
+        <v>145</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>66</v>
+        <v>146</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>67</v>
+        <v>147</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>68</v>
+        <v>148</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>69</v>
+        <v>149</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>70</v>
+        <v>150</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>71</v>
+        <v>151</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>72</v>
+        <v>152</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>73</v>
+        <v>153</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>74</v>
+        <v>154</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>75</v>
+        <v>155</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>76</v>
+        <v>156</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>77</v>
+        <v>157</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>78</v>
+        <v>158</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>79</v>
+        <v>159</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>80</v>
+        <v>160</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>81</v>
+        <v>161</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>82</v>
+        <v>162</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>83</v>
+        <v>163</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>84</v>
+        <v>164</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>85</v>
+        <v>165</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>86</v>
+        <v>166</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>87</v>
+        <v>167</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>88</v>
+        <v>168</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>89</v>
+        <v>169</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>90</v>
+        <v>170</v>
       </c>
       <c r="AF1" s="1" t="s">
-        <v>91</v>
+        <v>171</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>92</v>
+        <v>172</v>
       </c>
       <c r="AH1" s="1" t="s">
-        <v>93</v>
+        <v>173</v>
       </c>
       <c r="AI1" s="1" t="s">
-        <v>94</v>
+        <v>174</v>
       </c>
       <c r="AJ1" s="1" t="s">
-        <v>95</v>
+        <v>175</v>
       </c>
       <c r="AK1" s="1" t="s">
-        <v>96</v>
+        <v>176</v>
       </c>
       <c r="AL1" s="1" t="s">
-        <v>97</v>
+        <v>177</v>
       </c>
       <c r="AM1" s="1" t="s">
-        <v>98</v>
+        <v>178</v>
       </c>
       <c r="AN1" s="1" t="s">
-        <v>99</v>
+        <v>179</v>
       </c>
       <c r="AO1" s="1" t="s">
-        <v>100</v>
+        <v>180</v>
       </c>
       <c r="AP1" s="1" t="s">
-        <v>101</v>
+        <v>181</v>
       </c>
       <c r="AQ1" s="1" t="s">
-        <v>102</v>
+        <v>182</v>
       </c>
       <c r="AR1" s="1" t="s">
-        <v>103</v>
+        <v>183</v>
       </c>
       <c r="AS1" s="1" t="s">
-        <v>104</v>
+        <v>184</v>
       </c>
       <c r="AT1" s="1" t="s">
-        <v>105</v>
+        <v>185</v>
       </c>
       <c r="AU1" s="1" t="s">
-        <v>106</v>
+        <v>186</v>
       </c>
       <c r="AV1" s="1" t="s">
-        <v>107</v>
+        <v>187</v>
       </c>
       <c r="AW1" s="1" t="s">
-        <v>108</v>
+        <v>188</v>
       </c>
       <c r="AX1" s="1" t="s">
-        <v>109</v>
+        <v>189</v>
       </c>
       <c r="AY1" s="1" t="s">
-        <v>110</v>
+        <v>190</v>
       </c>
       <c r="AZ1" s="1" t="s">
-        <v>111</v>
+        <v>191</v>
       </c>
       <c r="BA1" s="1" t="s">
-        <v>112</v>
+        <v>192</v>
       </c>
     </row>
     <row r="29" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C29" s="2"/>
+      <c r="C29" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1370,22 +2526,22 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>36</v>
+        <v>116</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>37</v>
+        <v>117</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>38</v>
+        <v>118</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>39</v>
+        <v>119</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>40</v>
+        <v>120</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>41</v>
+        <v>121</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>2</v>
@@ -1397,13 +2553,13 @@
         <v>4</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>42</v>
+        <v>122</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>34</v>
+        <v>114</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>23</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -1413,32 +2569,6 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1453,22 +2583,72 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>46</v>
+        <v>126</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>47</v>
+        <v>127</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>48</v>
+        <v>128</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>43</v>
+        <v>123</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>44</v>
+        <v>124</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>45</v>
+        <v>125</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update production_system_intake.xlsx with new version. This should have the delivery dates and such. I am swstill working on the schedule/shift/OT tables etc. But this should be able to get us up and running.
</commit_message>
<xml_diff>
--- a/production_system_intake.xlsx
+++ b/production_system_intake.xlsx
@@ -5,38 +5,46 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Classes\2025_01_Spring\ASU\Computation\Week04\New folder\Intake\V04\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Classes\2025_01_Spring\ASU\Computation\Week04\New folder\Intake\V05\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA4AEF3C-A0C9-4474-ADED-D4BD4162BD77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36DF7E67-A7E1-4845-9223-D5CC07942245}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="2130" windowWidth="29040" windowHeight="15840" tabRatio="857" firstSheet="5" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="857" firstSheet="1" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProcessorTypeTbl" sheetId="3" r:id="rId1"/>
     <sheet name="LocationTbl" sheetId="4" r:id="rId2"/>
-    <sheet name="ProcessorTbl" sheetId="5" r:id="rId3"/>
-    <sheet name="TaskTbl" sheetId="1" r:id="rId4"/>
+    <sheet name="TaskTbl" sheetId="1" r:id="rId3"/>
+    <sheet name="TaskResourcesTbl" sheetId="18" r:id="rId4"/>
     <sheet name="ResourceTbl" sheetId="2" r:id="rId5"/>
-    <sheet name="TaskResourcesTbl" sheetId="18" r:id="rId6"/>
+    <sheet name="ProcessorTbl" sheetId="5" r:id="rId6"/>
     <sheet name="StationTbl" sheetId="6" r:id="rId7"/>
-    <sheet name="ConfigTbl" sheetId="8" r:id="rId8"/>
-    <sheet name="ProcessUnitTbl" sheetId="9" r:id="rId9"/>
-    <sheet name="ArrivalUnitTbl" sheetId="10" r:id="rId10"/>
-    <sheet name="ComponentsTbl" sheetId="11" r:id="rId11"/>
-    <sheet name="ProductsTbl" sheetId="7" r:id="rId12"/>
+    <sheet name="ProductsTbl" sheetId="7" r:id="rId8"/>
+    <sheet name="ConfigTbl" sheetId="8" r:id="rId9"/>
+    <sheet name="ProcessUnitTbl" sheetId="9" r:id="rId10"/>
+    <sheet name="ArrivalUnitTbl" sheetId="10" r:id="rId11"/>
+    <sheet name="ComponentsTbl" sheetId="11" r:id="rId12"/>
     <sheet name="Product01" sheetId="13" r:id="rId13"/>
-    <sheet name="ArrivalRatesTbl" sheetId="14" r:id="rId14"/>
-    <sheet name="ArrivalDatesTbl" sheetId="15" r:id="rId15"/>
+    <sheet name="ArrivalDatesTbl" sheetId="15" r:id="rId14"/>
+    <sheet name="ArrivalRatesTbl" sheetId="14" r:id="rId15"/>
     <sheet name="DeliveryRatesTbl" sheetId="16" r:id="rId16"/>
     <sheet name="DeliveryDatesTbl" sheetId="17" r:id="rId17"/>
+    <sheet name="PersonnelTbl_todo" sheetId="19" r:id="rId18"/>
+    <sheet name="HolidayClndrTbl_todo" sheetId="22" r:id="rId19"/>
+    <sheet name="PTOTbl_todo" sheetId="24" r:id="rId20"/>
+    <sheet name="OvertimeTable_todo" sheetId="25" r:id="rId21"/>
+    <sheet name="SchdPaternTbl_todo" sheetId="23" r:id="rId22"/>
+    <sheet name="ShiftTbl_todo" sheetId="20" r:id="rId23"/>
+    <sheet name="ShiftSegmentTbl_todo" sheetId="26" r:id="rId24"/>
+    <sheet name="ProductionModel_todo" sheetId="21" r:id="rId25"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="233">
   <si>
     <t>TaskIndex</t>
   </si>
@@ -332,6 +340,9 @@
     <t>ResourceIndex</t>
   </si>
   <si>
+    <t>ResourceIndex.1</t>
+  </si>
+  <si>
     <t>ResourceName</t>
   </si>
   <si>
@@ -620,7 +631,16 @@
     <t>TaskPred</t>
   </si>
   <si>
-    <t>ResourceID</t>
+    <t>ArrivalDate</t>
+  </si>
+  <si>
+    <t>ArrivalValue</t>
+  </si>
+  <si>
+    <t>ArrivalCount</t>
+  </si>
+  <si>
+    <t>ArrivalUnits</t>
   </si>
   <si>
     <t>ArrivalDatesIndex</t>
@@ -632,27 +652,15 @@
     <t>ArrivalDatesDesc</t>
   </si>
   <si>
-    <t>ArrivalDate</t>
-  </si>
-  <si>
-    <t>ArrivalCount</t>
+    <t>ArrivalRatesID</t>
   </si>
   <si>
     <t>ArrivalRatesIndex</t>
   </si>
   <si>
-    <t>ArrivalRatesID</t>
-  </si>
-  <si>
     <t>ArrivalRatesDesc</t>
   </si>
   <si>
-    <t>ArrivalValue</t>
-  </si>
-  <si>
-    <t>ArrivalUnits</t>
-  </si>
-  <si>
     <t>DeliveryRatesIndex</t>
   </si>
   <si>
@@ -662,19 +670,85 @@
     <t>DeliveryRatesDesc</t>
   </si>
   <si>
+    <t>DeliveryRateValue</t>
+  </si>
+  <si>
+    <t>DeliveryUnits</t>
+  </si>
+  <si>
+    <t>DeliveryCount</t>
+  </si>
+  <si>
     <t>DeliveryRateDate</t>
   </si>
   <si>
-    <t>DeliveryCount</t>
+    <t>PersonnelIndex</t>
+  </si>
+  <si>
+    <t>PersonnelID</t>
+  </si>
+  <si>
+    <t>PersonnelDesc</t>
+  </si>
+  <si>
+    <t>Npersonnel</t>
+  </si>
+  <si>
+    <t>ProductionRate</t>
+  </si>
+  <si>
+    <t>HourlyRate</t>
+  </si>
+  <si>
+    <t>Capacity</t>
+  </si>
+  <si>
+    <t>Schedual</t>
+  </si>
+  <si>
+    <t>Shift</t>
+  </si>
+  <si>
+    <t>HolidayCalendar</t>
+  </si>
+  <si>
+    <t>PTO</t>
+  </si>
+  <si>
+    <t>PTORate</t>
+  </si>
+  <si>
+    <t>OvertimeAllowance</t>
+  </si>
+  <si>
+    <t>OvertimeRate</t>
+  </si>
+  <si>
+    <t>OvertimeR</t>
+  </si>
+  <si>
+    <t>OnTimeStartReliability</t>
+  </si>
+  <si>
+    <t>OnTimeStartFailureDelay</t>
+  </si>
+  <si>
+    <t>ShiftIndex</t>
+  </si>
+  <si>
+    <t>ShiftID</t>
+  </si>
+  <si>
+    <t>ShiftDesc</t>
+  </si>
+  <si>
+    <t>ShiftTbl</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
-  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -743,13 +817,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1057,18 +1131,18 @@
   <cols>
     <col min="1" max="1" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -1077,13 +1151,13 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
@@ -1094,31 +1168,31 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>134</v>
-      </c>
       <c r="D1" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -1127,6 +1201,56 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:M1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1147,69 +1271,43 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="M1" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -1227,7 +1325,7 @@
   <sheetData>
     <row r="1" spans="1:81" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B1" t="s">
         <v>17</v>
@@ -1876,80 +1974,18 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
-  <dimension ref="A1:L1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.7109375" customWidth="1"/>
     <col min="5" max="5" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12" bestFit="1" customWidth="1"/>
@@ -1957,22 +1993,84 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>195</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D2" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
+  <dimension ref="A1:L1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.28515625" customWidth="1"/>
+    <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>203</v>
+      </c>
       <c r="B1" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>197</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>132</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>133</v>
@@ -1981,13 +2079,16 @@
         <v>134</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>124</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>125</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -1997,20 +2098,21 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>205</v>
       </c>
@@ -2023,17 +2125,20 @@
       <c r="D1" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>209</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>123</v>
+        <v>210</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>124</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>125</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -2047,9 +2152,9 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -2067,26 +2172,112 @@
         <v>207</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="2"/>
+      <c r="D2" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D8A8D90-B9D8-4E8E-B8C5-B87B3EDD59F1}">
+  <dimension ref="A1:Q1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="22" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>212</v>
+      </c>
+      <c r="B1" t="s">
+        <v>213</v>
+      </c>
+      <c r="C1" t="s">
+        <v>214</v>
+      </c>
+      <c r="D1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" t="s">
+        <v>216</v>
+      </c>
+      <c r="F1" t="s">
+        <v>217</v>
+      </c>
+      <c r="G1" t="s">
+        <v>218</v>
+      </c>
+      <c r="H1" t="s">
+        <v>219</v>
+      </c>
+      <c r="I1" t="s">
+        <v>220</v>
+      </c>
+      <c r="J1" t="s">
+        <v>221</v>
+      </c>
+      <c r="K1" t="s">
+        <v>222</v>
+      </c>
+      <c r="L1" t="s">
+        <v>223</v>
+      </c>
+      <c r="M1" t="s">
+        <v>227</v>
+      </c>
+      <c r="N1" t="s">
+        <v>228</v>
+      </c>
+      <c r="O1" t="s">
+        <v>224</v>
+      </c>
+      <c r="P1" t="s">
+        <v>225</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>226</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE4E35F8-7819-4E55-92CB-94AF21738FD2}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -2097,22 +2288,22 @@
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -2121,84 +2312,92 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:M1"/>
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDA296F8-8227-499C-B3D4-F942CBC18395}">
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="23" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.28515625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>115</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACFD5419-A74B-4CF2-B296-169B0EC9795C}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22DCE508-4EF3-4CE2-915A-C48C27323B08}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18FE2BAD-419E-4653-8809-5C67056F6E86}">
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>229</v>
+      </c>
+      <c r="B1" t="s">
+        <v>230</v>
+      </c>
+      <c r="C1" t="s">
+        <v>231</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{168A7E86-413A-43BD-B30E-2B11419D635F}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6CB75DA-14D0-47FB-91BA-328CDFE34017}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="79.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="30.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="20.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="19.42578125" bestFit="1" customWidth="1"/>
@@ -2221,7 +2420,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -2270,7 +2469,188 @@
       </c>
     </row>
     <row r="29" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C29" s="3"/>
+      <c r="C29" s="2"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E098E04-19A8-4E79-81CD-069FB2C95590}">
+  <dimension ref="A1:BA29"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="79.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="53" width="12.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:53" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="AL1" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="AN1" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="AO1" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="AP1" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="AQ1" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="AR1" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="AS1" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="AT1" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="AU1" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="AV1" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="AW1" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="AX1" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="AY1" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="AZ1" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="BA1" s="1" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="29" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C29" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -2284,13 +2664,13 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="27.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="23.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2298,25 +2678,25 @@
         <v>97</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>194</v>
+        <v>98</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -2325,179 +2705,65 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E098E04-19A8-4E79-81CD-069FB2C95590}">
-  <dimension ref="A1:BA29"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:M1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="53" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:53" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>142</v>
+        <v>4</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>143</v>
+        <v>105</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>144</v>
+        <v>106</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>145</v>
+        <v>107</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>146</v>
+        <v>112</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>147</v>
+        <v>108</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>148</v>
+        <v>109</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>149</v>
+        <v>113</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>150</v>
+        <v>114</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>151</v>
+        <v>115</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="AC1" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="AD1" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="AE1" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="AH1" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="AI1" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="AK1" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="AL1" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="AM1" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="AN1" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="AO1" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="AP1" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AQ1" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="AR1" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="AS1" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="AT1" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="AU1" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="AV1" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="AW1" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="AX1" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="AY1" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="AZ1" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="BA1" s="1" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="29" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C29" s="3"/>
+        <v>116</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -2512,36 +2778,36 @@
   <cols>
     <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="43.5703125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="22" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>2</v>
@@ -2553,13 +2819,13 @@
         <v>4</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -2569,6 +2835,32 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2577,78 +2869,26 @@
     <col min="2" max="2" width="8.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:I1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated intake and example. I have addate personnel andholday calendar and I am still workign on shift and scheduael planning more to come in the next few days. Then ingenstion will be the focus
</commit_message>
<xml_diff>
--- a/production_system_intake.xlsx
+++ b/production_system_intake.xlsx
@@ -5,20 +5,20 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Classes\2025_01_Spring\ASU\Computation\Week04\New folder\Intake\V05\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Classes\2025_01_Spring\ASU\Computation\Week03\Project\Dev\CAS502Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36DF7E67-A7E1-4845-9223-D5CC07942245}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{633EAAB9-C0C0-4D14-88A6-B4274DCF2F65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="857" firstSheet="1" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="2130" windowWidth="29040" windowHeight="15840" tabRatio="857" firstSheet="9" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProcessorTypeTbl" sheetId="3" r:id="rId1"/>
-    <sheet name="LocationTbl" sheetId="4" r:id="rId2"/>
-    <sheet name="TaskTbl" sheetId="1" r:id="rId3"/>
-    <sheet name="TaskResourcesTbl" sheetId="18" r:id="rId4"/>
-    <sheet name="ResourceTbl" sheetId="2" r:id="rId5"/>
-    <sheet name="ProcessorTbl" sheetId="5" r:id="rId6"/>
+    <sheet name="ProcessorTbl" sheetId="5" r:id="rId2"/>
+    <sheet name="LocationTbl" sheetId="4" r:id="rId3"/>
+    <sheet name="TaskTbl" sheetId="1" r:id="rId4"/>
+    <sheet name="TaskResourcesTbl" sheetId="18" r:id="rId5"/>
+    <sheet name="ResourceTbl" sheetId="2" r:id="rId6"/>
     <sheet name="StationTbl" sheetId="6" r:id="rId7"/>
     <sheet name="ProductsTbl" sheetId="7" r:id="rId8"/>
     <sheet name="ConfigTbl" sheetId="8" r:id="rId9"/>
@@ -30,21 +30,30 @@
     <sheet name="ArrivalRatesTbl" sheetId="14" r:id="rId15"/>
     <sheet name="DeliveryRatesTbl" sheetId="16" r:id="rId16"/>
     <sheet name="DeliveryDatesTbl" sheetId="17" r:id="rId17"/>
-    <sheet name="PersonnelTbl_todo" sheetId="19" r:id="rId18"/>
-    <sheet name="HolidayClndrTbl_todo" sheetId="22" r:id="rId19"/>
-    <sheet name="PTOTbl_todo" sheetId="24" r:id="rId20"/>
-    <sheet name="OvertimeTable_todo" sheetId="25" r:id="rId21"/>
-    <sheet name="SchdPaternTbl_todo" sheetId="23" r:id="rId22"/>
-    <sheet name="ShiftTbl_todo" sheetId="20" r:id="rId23"/>
-    <sheet name="ShiftSegmentTbl_todo" sheetId="26" r:id="rId24"/>
-    <sheet name="ProductionModel_todo" sheetId="21" r:id="rId25"/>
+    <sheet name="HolidayClndrTbl" sheetId="22" r:id="rId18"/>
+    <sheet name="PersonnelTbl" sheetId="19" r:id="rId19"/>
+    <sheet name="SchdPaternTbl_todo" sheetId="23" r:id="rId20"/>
+    <sheet name="ShiftTbl_todo" sheetId="20" r:id="rId21"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="234">
   <si>
     <t>TaskIndex</t>
   </si>
@@ -91,9 +100,6 @@
     <t>UnbatchingSize</t>
   </si>
   <si>
-    <t>UnbatchedSize</t>
-  </si>
-  <si>
     <t>ComponentsGenerated</t>
   </si>
   <si>
@@ -340,9 +346,6 @@
     <t>ResourceIndex</t>
   </si>
   <si>
-    <t>ResourceIndex.1</t>
-  </si>
-  <si>
     <t>ResourceName</t>
   </si>
   <si>
@@ -388,9 +391,6 @@
     <t>Location</t>
   </si>
   <si>
-    <t>DownProabilityPerUnity</t>
-  </si>
-  <si>
     <t>DownDelay</t>
   </si>
   <si>
@@ -703,30 +703,12 @@
     <t>Capacity</t>
   </si>
   <si>
-    <t>Schedual</t>
-  </si>
-  <si>
-    <t>Shift</t>
-  </si>
-  <si>
-    <t>HolidayCalendar</t>
-  </si>
-  <si>
-    <t>PTO</t>
-  </si>
-  <si>
-    <t>PTORate</t>
-  </si>
-  <si>
     <t>OvertimeAllowance</t>
   </si>
   <si>
     <t>OvertimeRate</t>
   </si>
   <si>
-    <t>OvertimeR</t>
-  </si>
-  <si>
     <t>OnTimeStartReliability</t>
   </si>
   <si>
@@ -742,14 +724,44 @@
     <t>ShiftDesc</t>
   </si>
   <si>
-    <t>ShiftTbl</t>
+    <t>task081</t>
+  </si>
+  <si>
+    <t>Pers001</t>
+  </si>
+  <si>
+    <t>Pers002</t>
+  </si>
+  <si>
+    <t>Pers003</t>
+  </si>
+  <si>
+    <t>Pers004</t>
+  </si>
+  <si>
+    <t>Pers005</t>
+  </si>
+  <si>
+    <t>PTOHrsAccrperWeek</t>
+  </si>
+  <si>
+    <t>PTOUtilizationRate</t>
+  </si>
+  <si>
+    <t>DelayUnits</t>
+  </si>
+  <si>
+    <t>HolidayBlackOutDates</t>
+  </si>
+  <si>
+    <t>ResourceID</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -774,6 +786,12 @@
       <u/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF141414"/>
+      <name val="Segoe UI"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -812,7 +830,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -824,6 +842,10 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1136,13 +1158,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>105</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -1168,31 +1190,31 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -1218,31 +1240,31 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -1256,58 +1278,57 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8.5703125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>142</v>
-      </c>
       <c r="H1" s="1" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -1317,655 +1338,714 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
-  <dimension ref="A1:CC81"/>
+  <dimension ref="A1:CD81"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="81" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="33.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15" bestFit="1" customWidth="1"/>
+    <col min="15" max="22" width="16" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="29" max="32" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="27" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="39" max="45" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="18" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="55" max="59" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="68" max="69" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="21" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="8" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="14.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:81" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:82" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>33</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>34</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>35</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>36</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>37</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>38</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>39</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>40</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>41</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>42</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" t="s">
         <v>43</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AD1" t="s">
         <v>44</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AE1" t="s">
         <v>45</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AF1" t="s">
         <v>46</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AG1" t="s">
         <v>47</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AH1" t="s">
         <v>48</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AI1" t="s">
         <v>49</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AJ1" t="s">
         <v>50</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AK1" t="s">
         <v>51</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AL1" t="s">
         <v>52</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AM1" t="s">
         <v>53</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AN1" t="s">
         <v>54</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AO1" t="s">
         <v>55</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AP1" t="s">
         <v>56</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AQ1" t="s">
         <v>57</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AR1" t="s">
         <v>58</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AS1" t="s">
         <v>59</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AT1" t="s">
         <v>60</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AU1" t="s">
         <v>61</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AV1" t="s">
         <v>62</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AW1" t="s">
         <v>63</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="AX1" t="s">
         <v>64</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="AY1" t="s">
         <v>65</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="AZ1" t="s">
         <v>66</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BA1" t="s">
         <v>67</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BB1" t="s">
         <v>68</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BC1" t="s">
         <v>69</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BD1" t="s">
         <v>70</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BE1" t="s">
         <v>71</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BF1" t="s">
         <v>72</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BG1" t="s">
         <v>73</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BH1" t="s">
         <v>74</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BI1" t="s">
         <v>75</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BJ1" t="s">
         <v>76</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BK1" t="s">
         <v>77</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BL1" t="s">
         <v>78</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BM1" t="s">
         <v>79</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BN1" t="s">
         <v>80</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BO1" t="s">
         <v>81</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BP1" t="s">
         <v>82</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="BQ1" t="s">
         <v>83</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="BR1" t="s">
         <v>84</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="BS1" t="s">
         <v>85</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="BT1" t="s">
         <v>86</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="BU1" t="s">
         <v>87</v>
       </c>
-      <c r="BU1" t="s">
+      <c r="BV1" t="s">
         <v>88</v>
       </c>
-      <c r="BV1" t="s">
+      <c r="BW1" t="s">
         <v>89</v>
       </c>
-      <c r="BW1" t="s">
+      <c r="BX1" t="s">
         <v>90</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="BY1" t="s">
         <v>91</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="BZ1" t="s">
         <v>92</v>
       </c>
-      <c r="BZ1" t="s">
+      <c r="CA1" t="s">
         <v>93</v>
       </c>
-      <c r="CA1" t="s">
+      <c r="CB1" t="s">
         <v>94</v>
       </c>
-      <c r="CB1" t="s">
+      <c r="CC1" t="s">
         <v>95</v>
       </c>
-      <c r="CC1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="2" spans="1:81" x14ac:dyDescent="0.25">
+      <c r="CD1" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="2" spans="1:82" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:82" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:81" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="4" spans="1:82" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:81" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="5" spans="1:82" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:81" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="6" spans="1:82" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:81" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="7" spans="1:82" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:81" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="8" spans="1:82" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:81" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="9" spans="1:82" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:81" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="10" spans="1:82" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:81" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="11" spans="1:82" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:81" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="12" spans="1:82" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:81" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="13" spans="1:82" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:81" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="14" spans="1:82" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:81" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="15" spans="1:82" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:81" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="16" spans="1:82" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>30</v>
-      </c>
-    </row>
-    <row r="16" spans="1:81" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -1975,7 +2055,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
@@ -1993,43 +2073,149 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D2" s="4"/>
     </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D3" s="4"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D4" s="4"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D5" s="4"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D6" s="4"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D7" s="4"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D8" s="4"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D9" s="4"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D10" s="4"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D11" s="4"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D12" s="4"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D13" s="4"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D14" s="4"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D15" s="4"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D16" s="4"/>
+    </row>
+    <row r="17" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D17" s="4"/>
+    </row>
+    <row r="18" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D18" s="4"/>
+    </row>
+    <row r="19" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D19" s="4"/>
+    </row>
+    <row r="20" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D20" s="4"/>
+    </row>
+    <row r="21" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D21" s="4"/>
+    </row>
+    <row r="22" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D22" s="4"/>
+    </row>
+    <row r="23" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D23" s="4"/>
+    </row>
+    <row r="24" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D24" s="4"/>
+    </row>
+    <row r="25" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D25" s="4"/>
+    </row>
+    <row r="26" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D26" s="4"/>
+    </row>
+    <row r="27" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D27" s="4"/>
+    </row>
+    <row r="28" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D28" s="4"/>
+    </row>
+    <row r="29" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D29" s="4"/>
+    </row>
+    <row r="30" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D30" s="4"/>
+    </row>
+    <row r="31" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D31" s="4"/>
+    </row>
+    <row r="32" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D32" s="4"/>
+    </row>
+    <row r="33" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D33" s="4"/>
+    </row>
+    <row r="34" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D34" s="4"/>
+    </row>
+    <row r="35" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D35" s="4"/>
+    </row>
+    <row r="36" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D36" s="4"/>
+    </row>
+    <row r="37" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D37" s="4"/>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2055,40 +2241,40 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -2114,31 +2300,31 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>210</v>
-      </c>
       <c r="G1" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -2163,28 +2349,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>210</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -2196,76 +2382,137 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D8A8D90-B9D8-4E8E-B8C5-B87B3EDD59F1}">
-  <dimension ref="A1:Q1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE4E35F8-7819-4E55-92CB-94AF21738FD2}">
+  <dimension ref="A1:A41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="22" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>212</v>
-      </c>
-      <c r="B1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C1" t="s">
-        <v>214</v>
-      </c>
-      <c r="D1" t="s">
-        <v>215</v>
-      </c>
-      <c r="E1" t="s">
-        <v>216</v>
-      </c>
-      <c r="F1" t="s">
-        <v>217</v>
-      </c>
-      <c r="G1" t="s">
-        <v>218</v>
-      </c>
-      <c r="H1" t="s">
-        <v>219</v>
-      </c>
-      <c r="I1" t="s">
-        <v>220</v>
-      </c>
-      <c r="J1" t="s">
-        <v>221</v>
-      </c>
-      <c r="K1" t="s">
-        <v>222</v>
-      </c>
-      <c r="L1" t="s">
-        <v>223</v>
-      </c>
-      <c r="M1" t="s">
-        <v>227</v>
-      </c>
-      <c r="N1" t="s">
-        <v>228</v>
-      </c>
-      <c r="O1" t="s">
-        <v>224</v>
-      </c>
-      <c r="P1" t="s">
-        <v>225</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>226</v>
-      </c>
+        <v>232</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="4"/>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4"/>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="4"/>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4"/>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4"/>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4"/>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4"/>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4"/>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4"/>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4"/>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" s="4"/>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="4"/>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="4"/>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="4"/>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="4"/>
+    </row>
+    <row r="17" spans="1:1" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A17" s="7"/>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="4"/>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4"/>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="4"/>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="4"/>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="4"/>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="4"/>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="4"/>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="4"/>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" s="4"/>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" s="4"/>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" s="4"/>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" s="4"/>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" s="4"/>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" s="4"/>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" s="4"/>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" s="4"/>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" s="4"/>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" s="4"/>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" s="4"/>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" s="4"/>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" s="4"/>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" s="4"/>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" s="4"/>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2273,438 +2520,133 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE4E35F8-7819-4E55-92CB-94AF21738FD2}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D8A8D90-B9D8-4E8E-B8C5-B87B3EDD59F1}">
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="11.85546875" customWidth="1"/>
+    <col min="5" max="6" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="22" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="19" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>209</v>
+      </c>
+      <c r="B1" t="s">
+        <v>210</v>
+      </c>
+      <c r="C1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" t="s">
+        <v>233</v>
+      </c>
+      <c r="E1" t="s">
+        <v>97</v>
+      </c>
+      <c r="F1" t="s">
+        <v>211</v>
+      </c>
+      <c r="G1" t="s">
+        <v>212</v>
+      </c>
+      <c r="H1" t="s">
+        <v>213</v>
+      </c>
+      <c r="I1" t="s">
+        <v>214</v>
+      </c>
+      <c r="J1" t="s">
+        <v>215</v>
+      </c>
+      <c r="K1" t="s">
+        <v>229</v>
+      </c>
+      <c r="L1" t="s">
+        <v>230</v>
+      </c>
+      <c r="M1" t="s">
+        <v>216</v>
+      </c>
+      <c r="N1" t="s">
+        <v>217</v>
+      </c>
+      <c r="O1" t="s">
+        <v>218</v>
+      </c>
+      <c r="P1" t="s">
+        <v>219</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>224</v>
+      </c>
+      <c r="L2" s="6"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>225</v>
+      </c>
+      <c r="L3" s="6"/>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>226</v>
+      </c>
+      <c r="L4" s="6"/>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>227</v>
+      </c>
+      <c r="L5" s="6"/>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>228</v>
+      </c>
+      <c r="L6" s="6"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.5703125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>111</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDA296F8-8227-499C-B3D4-F942CBC18395}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACFD5419-A74B-4CF2-B296-169B0EC9795C}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22DCE508-4EF3-4CE2-915A-C48C27323B08}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18FE2BAD-419E-4653-8809-5C67056F6E86}">
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>229</v>
-      </c>
-      <c r="B1" t="s">
-        <v>230</v>
-      </c>
-      <c r="C1" t="s">
-        <v>231</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{168A7E86-413A-43BD-B30E-2B11419D635F}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>232</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6CB75DA-14D0-47FB-91BA-328CDFE34017}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R29"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="79.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="30.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="22.28515625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="29" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C29" s="2"/>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E098E04-19A8-4E79-81CD-069FB2C95590}">
-  <dimension ref="A1:BA29"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="79.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="53" width="12.5703125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:53" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="AC1" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="AD1" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="AE1" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="AH1" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="AI1" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="AK1" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="AL1" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="AM1" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="AN1" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="AO1" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="AP1" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="AQ1" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="AR1" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="AS1" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="AT1" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="AU1" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="AV1" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="AW1" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="AX1" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="AY1" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="AZ1" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="BA1" s="1" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="29" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C29" s="2"/>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>104</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:M1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2735,38 +2677,1395 @@
         <v>4</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="J1" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="J1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>113</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>116</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22DCE508-4EF3-4CE2-915A-C48C27323B08}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18FE2BAD-419E-4653-8809-5C67056F6E86}">
+  <dimension ref="A1:II1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:243" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>220</v>
+      </c>
+      <c r="B1" t="s">
+        <v>221</v>
+      </c>
+      <c r="C1" t="s">
+        <v>222</v>
+      </c>
+      <c r="D1" s="8">
+        <v>0</v>
+      </c>
+      <c r="E1" s="8">
+        <v>4.1666666666666666E-3</v>
+      </c>
+      <c r="F1" s="8">
+        <v>8.3333333333333297E-3</v>
+      </c>
+      <c r="G1" s="8">
+        <v>1.2500000000000001E-2</v>
+      </c>
+      <c r="H1" s="8">
+        <v>1.6666666666666701E-2</v>
+      </c>
+      <c r="I1" s="8">
+        <v>2.0833333333333301E-2</v>
+      </c>
+      <c r="J1" s="8">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="K1" s="8">
+        <v>2.9166666666666698E-2</v>
+      </c>
+      <c r="L1" s="8">
+        <v>3.3333333333333298E-2</v>
+      </c>
+      <c r="M1" s="8">
+        <v>3.7499999999999999E-2</v>
+      </c>
+      <c r="N1" s="8">
+        <v>4.1666666666666699E-2</v>
+      </c>
+      <c r="O1" s="8">
+        <v>4.5833333333333302E-2</v>
+      </c>
+      <c r="P1" s="8">
+        <v>0.05</v>
+      </c>
+      <c r="Q1" s="8">
+        <v>5.4166666666666703E-2</v>
+      </c>
+      <c r="R1" s="8">
+        <v>5.83333333333333E-2</v>
+      </c>
+      <c r="S1" s="8">
+        <v>6.25E-2</v>
+      </c>
+      <c r="T1" s="8">
+        <v>6.6666666666666693E-2</v>
+      </c>
+      <c r="U1" s="8">
+        <v>7.0833333333333304E-2</v>
+      </c>
+      <c r="V1" s="8">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="W1" s="8">
+        <v>7.9166666666666705E-2</v>
+      </c>
+      <c r="X1" s="8">
+        <v>8.3333333333333301E-2</v>
+      </c>
+      <c r="Y1" s="8">
+        <v>8.7499999999999994E-2</v>
+      </c>
+      <c r="Z1" s="8">
+        <v>9.1666666666666702E-2</v>
+      </c>
+      <c r="AA1" s="8">
+        <v>9.5833333333333298E-2</v>
+      </c>
+      <c r="AB1" s="8">
+        <v>0.1</v>
+      </c>
+      <c r="AC1" s="8">
+        <v>0.104166666666667</v>
+      </c>
+      <c r="AD1" s="8">
+        <v>0.108333333333333</v>
+      </c>
+      <c r="AE1" s="8">
+        <v>0.1125</v>
+      </c>
+      <c r="AF1" s="8">
+        <v>0.116666666666667</v>
+      </c>
+      <c r="AG1" s="8">
+        <v>0.120833333333333</v>
+      </c>
+      <c r="AH1" s="8">
+        <v>0.125</v>
+      </c>
+      <c r="AI1" s="8">
+        <v>0.12916666666666701</v>
+      </c>
+      <c r="AJ1" s="8">
+        <v>0.133333333333333</v>
+      </c>
+      <c r="AK1" s="8">
+        <v>0.13750000000000001</v>
+      </c>
+      <c r="AL1" s="8">
+        <v>0.141666666666667</v>
+      </c>
+      <c r="AM1" s="8">
+        <v>0.14583333333333301</v>
+      </c>
+      <c r="AN1" s="8">
+        <v>0.15</v>
+      </c>
+      <c r="AO1" s="8">
+        <v>0.15416666666666701</v>
+      </c>
+      <c r="AP1" s="8">
+        <v>0.15833333333333299</v>
+      </c>
+      <c r="AQ1" s="8">
+        <v>0.16250000000000001</v>
+      </c>
+      <c r="AR1" s="8">
+        <v>0.16666666666666699</v>
+      </c>
+      <c r="AS1" s="8">
+        <v>0.170833333333333</v>
+      </c>
+      <c r="AT1" s="8">
+        <v>0.17499999999999999</v>
+      </c>
+      <c r="AU1" s="8">
+        <v>0.179166666666667</v>
+      </c>
+      <c r="AV1" s="8">
+        <v>0.18333333333333299</v>
+      </c>
+      <c r="AW1" s="8">
+        <v>0.1875</v>
+      </c>
+      <c r="AX1" s="8">
+        <v>0.19166666666666701</v>
+      </c>
+      <c r="AY1" s="8">
+        <v>0.195833333333333</v>
+      </c>
+      <c r="AZ1" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="BA1" s="8">
+        <v>0.204166666666667</v>
+      </c>
+      <c r="BB1" s="8">
+        <v>0.20833333333333301</v>
+      </c>
+      <c r="BC1" s="8">
+        <v>0.21249999999999999</v>
+      </c>
+      <c r="BD1" s="8">
+        <v>0.21666666666666701</v>
+      </c>
+      <c r="BE1" s="8">
+        <v>0.22083333333333299</v>
+      </c>
+      <c r="BF1" s="8">
+        <v>0.22500000000000001</v>
+      </c>
+      <c r="BG1" s="8">
+        <v>0.22916666666666699</v>
+      </c>
+      <c r="BH1" s="8">
+        <v>0.233333333333333</v>
+      </c>
+      <c r="BI1" s="8">
+        <v>0.23749999999999999</v>
+      </c>
+      <c r="BJ1" s="8">
+        <v>0.241666666666667</v>
+      </c>
+      <c r="BK1" s="8">
+        <v>0.24583333333333299</v>
+      </c>
+      <c r="BL1" s="8">
+        <v>0.25</v>
+      </c>
+      <c r="BM1" s="8">
+        <v>0.25416666666666698</v>
+      </c>
+      <c r="BN1" s="8">
+        <v>0.25833333333333303</v>
+      </c>
+      <c r="BO1" s="8">
+        <v>0.26250000000000001</v>
+      </c>
+      <c r="BP1" s="8">
+        <v>0.266666666666667</v>
+      </c>
+      <c r="BQ1" s="8">
+        <v>0.27083333333333298</v>
+      </c>
+      <c r="BR1" s="8">
+        <v>0.27500000000000002</v>
+      </c>
+      <c r="BS1" s="8">
+        <v>0.27916666666666701</v>
+      </c>
+      <c r="BT1" s="8">
+        <v>0.28333333333333299</v>
+      </c>
+      <c r="BU1" s="8">
+        <v>0.28749999999999998</v>
+      </c>
+      <c r="BV1" s="8">
+        <v>0.29166666666666702</v>
+      </c>
+      <c r="BW1" s="8">
+        <v>0.295833333333333</v>
+      </c>
+      <c r="BX1" s="8">
+        <v>0.3</v>
+      </c>
+      <c r="BY1" s="8">
+        <v>0.30416666666666697</v>
+      </c>
+      <c r="BZ1" s="8">
+        <v>0.30833333333333302</v>
+      </c>
+      <c r="CA1" s="8">
+        <v>0.3125</v>
+      </c>
+      <c r="CB1" s="8">
+        <v>0.31666666666666698</v>
+      </c>
+      <c r="CC1" s="8">
+        <v>0.32083333333333303</v>
+      </c>
+      <c r="CD1" s="8">
+        <v>0.32500000000000001</v>
+      </c>
+      <c r="CE1" s="8">
+        <v>0.329166666666667</v>
+      </c>
+      <c r="CF1" s="8">
+        <v>0.33333333333333298</v>
+      </c>
+      <c r="CG1" s="8">
+        <v>0.33750000000000002</v>
+      </c>
+      <c r="CH1" s="8">
+        <v>0.34166666666666701</v>
+      </c>
+      <c r="CI1" s="8">
+        <v>0.34583333333333299</v>
+      </c>
+      <c r="CJ1" s="8">
+        <v>0.35</v>
+      </c>
+      <c r="CK1" s="8">
+        <v>0.35416666666666702</v>
+      </c>
+      <c r="CL1" s="8">
+        <v>0.358333333333333</v>
+      </c>
+      <c r="CM1" s="8">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="CN1" s="8">
+        <v>0.36666666666666697</v>
+      </c>
+      <c r="CO1" s="8">
+        <v>0.37083333333333302</v>
+      </c>
+      <c r="CP1" s="8">
+        <v>0.375</v>
+      </c>
+      <c r="CQ1" s="8">
+        <v>0.37916666666666698</v>
+      </c>
+      <c r="CR1" s="8">
+        <v>0.38333333333333303</v>
+      </c>
+      <c r="CS1" s="8">
+        <v>0.38750000000000001</v>
+      </c>
+      <c r="CT1" s="8">
+        <v>0.391666666666667</v>
+      </c>
+      <c r="CU1" s="8">
+        <v>0.39583333333333298</v>
+      </c>
+      <c r="CV1" s="8">
+        <v>0.4</v>
+      </c>
+      <c r="CW1" s="8">
+        <v>0.40416666666666701</v>
+      </c>
+      <c r="CX1" s="8">
+        <v>0.40833333333333299</v>
+      </c>
+      <c r="CY1" s="8">
+        <v>0.41249999999999998</v>
+      </c>
+      <c r="CZ1" s="8">
+        <v>0.41666666666666702</v>
+      </c>
+      <c r="DA1" s="8">
+        <v>0.420833333333333</v>
+      </c>
+      <c r="DB1" s="8">
+        <v>0.42499999999999999</v>
+      </c>
+      <c r="DC1" s="8">
+        <v>0.42916666666666697</v>
+      </c>
+      <c r="DD1" s="8">
+        <v>0.43333333333333302</v>
+      </c>
+      <c r="DE1" s="8">
+        <v>0.4375</v>
+      </c>
+      <c r="DF1" s="8">
+        <v>0.44166666666666698</v>
+      </c>
+      <c r="DG1" s="8">
+        <v>0.44583333333333303</v>
+      </c>
+      <c r="DH1" s="8">
+        <v>0.45</v>
+      </c>
+      <c r="DI1" s="8">
+        <v>0.454166666666667</v>
+      </c>
+      <c r="DJ1" s="8">
+        <v>0.45833333333333298</v>
+      </c>
+      <c r="DK1" s="8">
+        <v>0.46250000000000002</v>
+      </c>
+      <c r="DL1" s="8">
+        <v>0.46666666666666701</v>
+      </c>
+      <c r="DM1" s="8">
+        <v>0.47083333333333299</v>
+      </c>
+      <c r="DN1" s="8">
+        <v>0.47499999999999998</v>
+      </c>
+      <c r="DO1" s="8">
+        <v>0.47916666666666702</v>
+      </c>
+      <c r="DP1" s="8">
+        <v>0.483333333333333</v>
+      </c>
+      <c r="DQ1" s="8">
+        <v>0.48749999999999999</v>
+      </c>
+      <c r="DR1" s="8">
+        <v>0.49166666666666697</v>
+      </c>
+      <c r="DS1" s="8">
+        <v>0.49583333333333302</v>
+      </c>
+      <c r="DT1" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="DU1" s="8">
+        <v>0.50416666666666698</v>
+      </c>
+      <c r="DV1" s="8">
+        <v>0.50833333333333297</v>
+      </c>
+      <c r="DW1" s="8">
+        <v>0.51249999999999996</v>
+      </c>
+      <c r="DX1" s="8">
+        <v>0.51666666666666705</v>
+      </c>
+      <c r="DY1" s="8">
+        <v>0.52083333333333304</v>
+      </c>
+      <c r="DZ1" s="8">
+        <v>0.52500000000000002</v>
+      </c>
+      <c r="EA1" s="8">
+        <v>0.52916666666666701</v>
+      </c>
+      <c r="EB1" s="8">
+        <v>0.53333333333333299</v>
+      </c>
+      <c r="EC1" s="8">
+        <v>0.53749999999999998</v>
+      </c>
+      <c r="ED1" s="8">
+        <v>0.54166666666666696</v>
+      </c>
+      <c r="EE1" s="8">
+        <v>0.54583333333333295</v>
+      </c>
+      <c r="EF1" s="8">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="EG1" s="8">
+        <v>0.55416666666666703</v>
+      </c>
+      <c r="EH1" s="8">
+        <v>0.55833333333333302</v>
+      </c>
+      <c r="EI1" s="8">
+        <v>0.5625</v>
+      </c>
+      <c r="EJ1" s="8">
+        <v>0.56666666666666698</v>
+      </c>
+      <c r="EK1" s="8">
+        <v>0.57083333333333297</v>
+      </c>
+      <c r="EL1" s="8">
+        <v>0.57499999999999996</v>
+      </c>
+      <c r="EM1" s="8">
+        <v>0.57916666666666705</v>
+      </c>
+      <c r="EN1" s="8">
+        <v>0.58333333333333304</v>
+      </c>
+      <c r="EO1" s="8">
+        <v>0.58750000000000002</v>
+      </c>
+      <c r="EP1" s="8">
+        <v>0.59166666666666701</v>
+      </c>
+      <c r="EQ1" s="8">
+        <v>0.59583333333333299</v>
+      </c>
+      <c r="ER1" s="8">
+        <v>0.6</v>
+      </c>
+      <c r="ES1" s="8">
+        <v>0.60416666666666696</v>
+      </c>
+      <c r="ET1" s="8">
+        <v>0.60833333333333295</v>
+      </c>
+      <c r="EU1" s="8">
+        <v>0.61250000000000004</v>
+      </c>
+      <c r="EV1" s="8">
+        <v>0.61666666666666703</v>
+      </c>
+      <c r="EW1" s="8">
+        <v>0.62083333333333302</v>
+      </c>
+      <c r="EX1" s="8">
+        <v>0.625</v>
+      </c>
+      <c r="EY1" s="8">
+        <v>0.62916666666666698</v>
+      </c>
+      <c r="EZ1" s="8">
+        <v>0.63333333333333297</v>
+      </c>
+      <c r="FA1" s="8">
+        <v>0.63749999999999996</v>
+      </c>
+      <c r="FB1" s="8">
+        <v>0.64166666666666705</v>
+      </c>
+      <c r="FC1" s="8">
+        <v>0.64583333333333304</v>
+      </c>
+      <c r="FD1" s="8">
+        <v>0.65</v>
+      </c>
+      <c r="FE1" s="8">
+        <v>0.65416666666666701</v>
+      </c>
+      <c r="FF1" s="8">
+        <v>0.65833333333333299</v>
+      </c>
+      <c r="FG1" s="8">
+        <v>0.66249999999999998</v>
+      </c>
+      <c r="FH1" s="8">
+        <v>0.66666666666666696</v>
+      </c>
+      <c r="FI1" s="8">
+        <v>0.67083333333333295</v>
+      </c>
+      <c r="FJ1" s="8">
+        <v>0.67500000000000004</v>
+      </c>
+      <c r="FK1" s="8">
+        <v>0.67916666666666703</v>
+      </c>
+      <c r="FL1" s="8">
+        <v>0.68333333333333302</v>
+      </c>
+      <c r="FM1" s="8">
+        <v>0.6875</v>
+      </c>
+      <c r="FN1" s="8">
+        <v>0.69166666666666698</v>
+      </c>
+      <c r="FO1" s="8">
+        <v>0.69583333333333297</v>
+      </c>
+      <c r="FP1" s="8">
+        <v>0.7</v>
+      </c>
+      <c r="FQ1" s="8">
+        <v>0.70416666666666705</v>
+      </c>
+      <c r="FR1" s="8">
+        <v>0.70833333333333304</v>
+      </c>
+      <c r="FS1" s="8">
+        <v>0.71250000000000002</v>
+      </c>
+      <c r="FT1" s="8">
+        <v>0.71666666666666701</v>
+      </c>
+      <c r="FU1" s="8">
+        <v>0.72083333333333299</v>
+      </c>
+      <c r="FV1" s="8">
+        <v>0.72499999999999998</v>
+      </c>
+      <c r="FW1" s="8">
+        <v>0.72916666666666696</v>
+      </c>
+      <c r="FX1" s="8">
+        <v>0.73333333333333295</v>
+      </c>
+      <c r="FY1" s="8">
+        <v>0.73750000000000004</v>
+      </c>
+      <c r="FZ1" s="8">
+        <v>0.74166666666666703</v>
+      </c>
+      <c r="GA1" s="8">
+        <v>0.74583333333333302</v>
+      </c>
+      <c r="GB1" s="8">
+        <v>0.75</v>
+      </c>
+      <c r="GC1" s="8">
+        <v>0.75416666666666698</v>
+      </c>
+      <c r="GD1" s="8">
+        <v>0.75833333333333297</v>
+      </c>
+      <c r="GE1" s="8">
+        <v>0.76249999999999996</v>
+      </c>
+      <c r="GF1" s="8">
+        <v>0.76666666666666705</v>
+      </c>
+      <c r="GG1" s="8">
+        <v>0.77083333333333304</v>
+      </c>
+      <c r="GH1" s="8">
+        <v>0.77500000000000002</v>
+      </c>
+      <c r="GI1" s="8">
+        <v>0.77916666666666701</v>
+      </c>
+      <c r="GJ1" s="8">
+        <v>0.78333333333333299</v>
+      </c>
+      <c r="GK1" s="8">
+        <v>0.78749999999999998</v>
+      </c>
+      <c r="GL1" s="8">
+        <v>0.79166666666666696</v>
+      </c>
+      <c r="GM1" s="8">
+        <v>0.79583333333333295</v>
+      </c>
+      <c r="GN1" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="GO1" s="8">
+        <v>0.80416666666666703</v>
+      </c>
+      <c r="GP1" s="8">
+        <v>0.80833333333333302</v>
+      </c>
+      <c r="GQ1" s="8">
+        <v>0.8125</v>
+      </c>
+      <c r="GR1" s="8">
+        <v>0.81666666666666698</v>
+      </c>
+      <c r="GS1" s="8">
+        <v>0.82083333333333297</v>
+      </c>
+      <c r="GT1" s="8">
+        <v>0.82499999999999996</v>
+      </c>
+      <c r="GU1" s="8">
+        <v>0.82916666666666705</v>
+      </c>
+      <c r="GV1" s="8">
+        <v>0.83333333333333304</v>
+      </c>
+      <c r="GW1" s="8">
+        <v>0.83750000000000002</v>
+      </c>
+      <c r="GX1" s="8">
+        <v>0.84166666666666701</v>
+      </c>
+      <c r="GY1" s="8">
+        <v>0.84583333333333299</v>
+      </c>
+      <c r="GZ1" s="8">
+        <v>0.85</v>
+      </c>
+      <c r="HA1" s="8">
+        <v>0.85416666666666696</v>
+      </c>
+      <c r="HB1" s="8">
+        <v>0.85833333333333295</v>
+      </c>
+      <c r="HC1" s="8">
+        <v>0.86250000000000004</v>
+      </c>
+      <c r="HD1" s="8">
+        <v>0.86666666666666703</v>
+      </c>
+      <c r="HE1" s="8">
+        <v>0.87083333333333302</v>
+      </c>
+      <c r="HF1" s="8">
+        <v>0.875</v>
+      </c>
+      <c r="HG1" s="8">
+        <v>0.87916666666666698</v>
+      </c>
+      <c r="HH1" s="8">
+        <v>0.88333333333333297</v>
+      </c>
+      <c r="HI1" s="8">
+        <v>0.88749999999999996</v>
+      </c>
+      <c r="HJ1" s="8">
+        <v>0.89166666666666705</v>
+      </c>
+      <c r="HK1" s="8">
+        <v>0.89583333333333304</v>
+      </c>
+      <c r="HL1" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="HM1" s="8">
+        <v>0.90416666666666701</v>
+      </c>
+      <c r="HN1" s="8">
+        <v>0.90833333333333299</v>
+      </c>
+      <c r="HO1" s="8">
+        <v>0.91249999999999998</v>
+      </c>
+      <c r="HP1" s="8">
+        <v>0.91666666666666696</v>
+      </c>
+      <c r="HQ1" s="8">
+        <v>0.92083333333333295</v>
+      </c>
+      <c r="HR1" s="8">
+        <v>0.92500000000000004</v>
+      </c>
+      <c r="HS1" s="8">
+        <v>0.92916666666666703</v>
+      </c>
+      <c r="HT1" s="8">
+        <v>0.93333333333333302</v>
+      </c>
+      <c r="HU1" s="8">
+        <v>0.9375</v>
+      </c>
+      <c r="HV1" s="8">
+        <v>0.94166666666666698</v>
+      </c>
+      <c r="HW1" s="8">
+        <v>0.94583333333333297</v>
+      </c>
+      <c r="HX1" s="8">
+        <v>0.95</v>
+      </c>
+      <c r="HY1" s="8">
+        <v>0.95416666666666705</v>
+      </c>
+      <c r="HZ1" s="8">
+        <v>0.95833333333333304</v>
+      </c>
+      <c r="IA1" s="8">
+        <v>0.96250000000000002</v>
+      </c>
+      <c r="IB1" s="8">
+        <v>0.96666666666666701</v>
+      </c>
+      <c r="IC1" s="8">
+        <v>0.97083333333333299</v>
+      </c>
+      <c r="ID1" s="8">
+        <v>0.97499999999999998</v>
+      </c>
+      <c r="IE1" s="8">
+        <v>0.97916666666666696</v>
+      </c>
+      <c r="IF1" s="8">
+        <v>0.98333333333333295</v>
+      </c>
+      <c r="IG1" s="8">
+        <v>0.98750000000000004</v>
+      </c>
+      <c r="IH1" s="8">
+        <v>0.99166666666666703</v>
+      </c>
+      <c r="II1" s="8">
+        <v>0.99583333333333302</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:Q82"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="79.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="30.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N2" s="5"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N3" s="5"/>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N4" s="5"/>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N5" s="5"/>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N6" s="5"/>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N7" s="5"/>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N8" s="5"/>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N9" s="5"/>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N10" s="5"/>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N11" s="5"/>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N12" s="5"/>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N13" s="5"/>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N14" s="5"/>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N15" s="5"/>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N16" s="5"/>
+    </row>
+    <row r="17" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="N17" s="5"/>
+    </row>
+    <row r="18" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="N18" s="5"/>
+    </row>
+    <row r="19" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="N19" s="5"/>
+    </row>
+    <row r="20" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="N20" s="5"/>
+    </row>
+    <row r="21" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="N21" s="5"/>
+    </row>
+    <row r="22" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="N22" s="5"/>
+    </row>
+    <row r="23" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="N23" s="5"/>
+    </row>
+    <row r="24" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="N24" s="5"/>
+    </row>
+    <row r="25" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="N25" s="5"/>
+    </row>
+    <row r="26" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="N26" s="5"/>
+    </row>
+    <row r="27" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="N27" s="5"/>
+    </row>
+    <row r="28" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="N28" s="5"/>
+    </row>
+    <row r="29" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="N29" s="5"/>
+    </row>
+    <row r="30" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="C30" s="2"/>
+      <c r="N30" s="5"/>
+    </row>
+    <row r="31" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="N31" s="5"/>
+    </row>
+    <row r="32" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="N32" s="5"/>
+    </row>
+    <row r="33" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N33" s="5"/>
+    </row>
+    <row r="34" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N34" s="5"/>
+    </row>
+    <row r="35" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N35" s="5"/>
+    </row>
+    <row r="36" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N36" s="5"/>
+    </row>
+    <row r="37" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N37" s="5"/>
+    </row>
+    <row r="38" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N38" s="5"/>
+    </row>
+    <row r="39" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N39" s="5"/>
+    </row>
+    <row r="40" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N40" s="5"/>
+    </row>
+    <row r="41" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N41" s="5"/>
+    </row>
+    <row r="42" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N42" s="5"/>
+    </row>
+    <row r="43" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N43" s="5"/>
+    </row>
+    <row r="44" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N44" s="5"/>
+    </row>
+    <row r="45" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N45" s="5"/>
+    </row>
+    <row r="46" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N46" s="5"/>
+    </row>
+    <row r="47" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N47" s="5"/>
+    </row>
+    <row r="48" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N48" s="5"/>
+    </row>
+    <row r="49" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N49" s="5"/>
+    </row>
+    <row r="50" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N50" s="5"/>
+    </row>
+    <row r="51" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N51" s="5"/>
+    </row>
+    <row r="52" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N52" s="5"/>
+    </row>
+    <row r="53" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N53" s="5"/>
+    </row>
+    <row r="54" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N54" s="5"/>
+    </row>
+    <row r="55" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N55" s="5"/>
+    </row>
+    <row r="56" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N56" s="5"/>
+    </row>
+    <row r="57" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N57" s="5"/>
+    </row>
+    <row r="58" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N58" s="5"/>
+    </row>
+    <row r="59" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N59" s="5"/>
+    </row>
+    <row r="60" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N60" s="5"/>
+    </row>
+    <row r="61" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N61" s="5"/>
+    </row>
+    <row r="62" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N62" s="5"/>
+    </row>
+    <row r="63" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N63" s="5"/>
+    </row>
+    <row r="64" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N64" s="5"/>
+    </row>
+    <row r="65" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N65" s="5"/>
+    </row>
+    <row r="66" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N66" s="5"/>
+    </row>
+    <row r="67" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N67" s="5"/>
+    </row>
+    <row r="68" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N68" s="5"/>
+    </row>
+    <row r="69" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N69" s="5"/>
+    </row>
+    <row r="70" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N70" s="5"/>
+    </row>
+    <row r="71" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N71" s="5"/>
+    </row>
+    <row r="72" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N72" s="5"/>
+    </row>
+    <row r="73" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N73" s="5"/>
+    </row>
+    <row r="74" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N74" s="5"/>
+    </row>
+    <row r="75" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N75" s="5"/>
+    </row>
+    <row r="76" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N76" s="5"/>
+    </row>
+    <row r="77" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N77" s="5"/>
+    </row>
+    <row r="78" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N78" s="5"/>
+    </row>
+    <row r="79" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N79" s="5"/>
+    </row>
+    <row r="80" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N80" s="5"/>
+    </row>
+    <row r="81" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N81" s="5"/>
+    </row>
+    <row r="82" spans="14:14" x14ac:dyDescent="0.25">
+      <c r="N82" s="5"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E098E04-19A8-4E79-81CD-069FB2C95590}">
+  <dimension ref="A1:BA30"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="79.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="19" max="25" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="27" max="28" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="33.140625" bestFit="1" customWidth="1"/>
+    <col min="32" max="53" width="12.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:53" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="AL1" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="AN1" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="AO1" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="AP1" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="AQ1" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="AR1" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="AS1" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="AT1" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="AU1" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="AV1" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="AW1" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="AX1" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="AY1" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="AZ1" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="BA1" s="1" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="30" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C30" s="2"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2777,7 +4076,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="41.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21.42578125" bestFit="1" customWidth="1"/>
@@ -2792,22 +4091,22 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>122</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>2</v>
@@ -2819,13 +4118,13 @@
         <v>4</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -2846,13 +4145,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -2873,22 +4172,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated Intakefiles. it took a long time but I finally developmed a model for presoneel, the shifts, scheduale, PTO, and holidays for the production system and I updated the example.
</commit_message>
<xml_diff>
--- a/production_system_intake.xlsx
+++ b/production_system_intake.xlsx
@@ -5,20 +5,20 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Classes\2025_01_Spring\ASU\Computation\Week03\Project\Dev\CAS502Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Classes\2025_01_Spring\ASU\Computation\Week03\Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{633EAAB9-C0C0-4D14-88A6-B4274DCF2F65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC18DDE-FC0A-41A7-8B57-58FC67BFF982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="2130" windowWidth="29040" windowHeight="15840" tabRatio="857" firstSheet="9" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="2130" windowWidth="29040" windowHeight="15840" tabRatio="857" firstSheet="9" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProcessorTypeTbl" sheetId="3" r:id="rId1"/>
-    <sheet name="ProcessorTbl" sheetId="5" r:id="rId2"/>
-    <sheet name="LocationTbl" sheetId="4" r:id="rId3"/>
-    <sheet name="TaskTbl" sheetId="1" r:id="rId4"/>
-    <sheet name="TaskResourcesTbl" sheetId="18" r:id="rId5"/>
-    <sheet name="ResourceTbl" sheetId="2" r:id="rId6"/>
+    <sheet name="LocationTbl" sheetId="4" r:id="rId2"/>
+    <sheet name="TaskTbl" sheetId="1" r:id="rId3"/>
+    <sheet name="TaskResourcesTbl" sheetId="18" r:id="rId4"/>
+    <sheet name="ResourceTbl" sheetId="2" r:id="rId5"/>
+    <sheet name="ProcessorTbl" sheetId="5" r:id="rId6"/>
     <sheet name="StationTbl" sheetId="6" r:id="rId7"/>
     <sheet name="ProductsTbl" sheetId="7" r:id="rId8"/>
     <sheet name="ConfigTbl" sheetId="8" r:id="rId9"/>
@@ -30,10 +30,11 @@
     <sheet name="ArrivalRatesTbl" sheetId="14" r:id="rId15"/>
     <sheet name="DeliveryRatesTbl" sheetId="16" r:id="rId16"/>
     <sheet name="DeliveryDatesTbl" sheetId="17" r:id="rId17"/>
-    <sheet name="HolidayClndrTbl" sheetId="22" r:id="rId18"/>
-    <sheet name="PersonnelTbl" sheetId="19" r:id="rId19"/>
-    <sheet name="SchdPaternTbl_todo" sheetId="23" r:id="rId20"/>
-    <sheet name="ShiftTbl_todo" sheetId="20" r:id="rId21"/>
+    <sheet name="PersonnelTbl" sheetId="19" r:id="rId18"/>
+    <sheet name="SchdPtrnTbl" sheetId="23" r:id="rId19"/>
+    <sheet name="ShiftTbl" sheetId="20" r:id="rId20"/>
+    <sheet name="HolidayClndrTbl" sheetId="22" r:id="rId21"/>
+    <sheet name="PTOTbl" sheetId="24" r:id="rId22"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -53,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="298">
   <si>
     <t>TaskIndex</t>
   </si>
@@ -346,6 +347,9 @@
     <t>ResourceIndex</t>
   </si>
   <si>
+    <t>ResourceIndex.1</t>
+  </si>
+  <si>
     <t>ResourceName</t>
   </si>
   <si>
@@ -364,6 +368,54 @@
     <t>Units</t>
   </si>
   <si>
+    <t>Quality Inspector</t>
+  </si>
+  <si>
+    <t>Mech Tech</t>
+  </si>
+  <si>
+    <t>Flotron</t>
+  </si>
+  <si>
+    <t>Panel Assmebly Stands</t>
+  </si>
+  <si>
+    <t>SV/Prop Lifting Sling</t>
+  </si>
+  <si>
+    <t>SV Lifting GS</t>
+  </si>
+  <si>
+    <t>TVAC Config GSE</t>
+  </si>
+  <si>
+    <t>Stack Lifting GSE</t>
+  </si>
+  <si>
+    <t>Dynamics Config GSE</t>
+  </si>
+  <si>
+    <t>Vacuum Chamber</t>
+  </si>
+  <si>
+    <t>Digital Multi Meter</t>
+  </si>
+  <si>
+    <t>Prop GSE</t>
+  </si>
+  <si>
+    <t>GPS Sim</t>
+  </si>
+  <si>
+    <t>Mass Prop GSE</t>
+  </si>
+  <si>
+    <t>Host Rack</t>
+  </si>
+  <si>
+    <t>Hardware Delivered from Inventory</t>
+  </si>
+  <si>
     <t>ProcessorTypeIndex</t>
   </si>
   <si>
@@ -385,12 +437,18 @@
     <t>AreaDesc</t>
   </si>
   <si>
+    <t>SQFT</t>
+  </si>
+  <si>
     <t>NumberStations</t>
   </si>
   <si>
     <t>Location</t>
   </si>
   <si>
+    <t>DownProabilityPerUnity</t>
+  </si>
+  <si>
     <t>DownDelay</t>
   </si>
   <si>
@@ -478,6 +536,45 @@
     <t>TasksDesc</t>
   </si>
   <si>
+    <t>Egnr</t>
+  </si>
+  <si>
+    <t>Tech</t>
+  </si>
+  <si>
+    <t>MI tech</t>
+  </si>
+  <si>
+    <t>Sys01 Rack</t>
+  </si>
+  <si>
+    <t>Sys02 Rack</t>
+  </si>
+  <si>
+    <t>Sys03 Rack</t>
+  </si>
+  <si>
+    <t>Sys04 Rack</t>
+  </si>
+  <si>
+    <t>Stimulator</t>
+  </si>
+  <si>
+    <t>Sys05 Rack</t>
+  </si>
+  <si>
+    <t>Sys06 rack</t>
+  </si>
+  <si>
+    <t>Sys07 Rack (traveler)</t>
+  </si>
+  <si>
+    <t>Sys00 Rack (Workcell)</t>
+  </si>
+  <si>
+    <t>SV w/ Panels</t>
+  </si>
+  <si>
     <t>NResource01</t>
   </si>
   <si>
@@ -703,6 +800,15 @@
     <t>Capacity</t>
   </si>
   <si>
+    <t>Schedual</t>
+  </si>
+  <si>
+    <t>Shift</t>
+  </si>
+  <si>
+    <t>HolidayCalendar</t>
+  </si>
+  <si>
     <t>OvertimeAllowance</t>
   </si>
   <si>
@@ -724,43 +830,133 @@
     <t>ShiftDesc</t>
   </si>
   <si>
-    <t>task081</t>
-  </si>
-  <si>
-    <t>Pers001</t>
-  </si>
-  <si>
-    <t>Pers002</t>
-  </si>
-  <si>
-    <t>Pers003</t>
-  </si>
-  <si>
-    <t>Pers004</t>
-  </si>
-  <si>
-    <t>Pers005</t>
-  </si>
-  <si>
-    <t>PTOHrsAccrperWeek</t>
-  </si>
-  <si>
-    <t>PTOUtilizationRate</t>
-  </si>
-  <si>
-    <t>DelayUnits</t>
-  </si>
-  <si>
-    <t>HolidayBlackOutDates</t>
-  </si>
-  <si>
-    <t>ResourceID</t>
+    <t>ShiftStart</t>
+  </si>
+  <si>
+    <t>ShiftBreakStart</t>
+  </si>
+  <si>
+    <t>ShiftBreakEnd</t>
+  </si>
+  <si>
+    <t>StartBuffer</t>
+  </si>
+  <si>
+    <t>EndBuffer</t>
+  </si>
+  <si>
+    <t>ShiftLength</t>
+  </si>
+  <si>
+    <t>ShiftStartUnit</t>
+  </si>
+  <si>
+    <t>ShiftEndUnit</t>
+  </si>
+  <si>
+    <t>ShiftEnd</t>
+  </si>
+  <si>
+    <t>ShiftBreakStartUnit</t>
+  </si>
+  <si>
+    <t>ShiftBreakEndUnit</t>
+  </si>
+  <si>
+    <t>TotalStaffingTime</t>
+  </si>
+  <si>
+    <t>BaseProductionTime</t>
+  </si>
+  <si>
+    <t>ProductionStartTimePart1</t>
+  </si>
+  <si>
+    <t>ProductionEndTimePart1</t>
+  </si>
+  <si>
+    <t>ProductionStartTimePart2</t>
+  </si>
+  <si>
+    <t>ProductionEndTimePart2</t>
+  </si>
+  <si>
+    <t>BreakLength</t>
+  </si>
+  <si>
+    <t>Day01</t>
+  </si>
+  <si>
+    <t>Day02</t>
+  </si>
+  <si>
+    <t>Day03</t>
+  </si>
+  <si>
+    <t>Day04</t>
+  </si>
+  <si>
+    <t>Day05</t>
+  </si>
+  <si>
+    <t>Day06</t>
+  </si>
+  <si>
+    <t>Day07</t>
+  </si>
+  <si>
+    <t>SchdPtrnIndex</t>
+  </si>
+  <si>
+    <t>SchdPtrnID</t>
+  </si>
+  <si>
+    <t>SchdPtrnDesc</t>
+  </si>
+  <si>
+    <t>ShiftStartDate</t>
+  </si>
+  <si>
+    <t>HolidayCalendar01</t>
+  </si>
+  <si>
+    <t>HolidayDays</t>
+  </si>
+  <si>
+    <t>PTOCalendar01</t>
+  </si>
+  <si>
+    <t>PTORatePerWeek</t>
+  </si>
+  <si>
+    <t>PTOUtilization</t>
+  </si>
+  <si>
+    <t>PTODay01</t>
+  </si>
+  <si>
+    <t>PTOYearlySum01</t>
+  </si>
+  <si>
+    <t>HolidayCalendarDay01</t>
+  </si>
+  <si>
+    <t>Year01</t>
+  </si>
+  <si>
+    <t>PTOYear01</t>
+  </si>
+  <si>
+    <t>PTOCalendar</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+  </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -789,9 +985,9 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF141414"/>
-      <name val="Segoe UI"/>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Verdana"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -830,7 +1026,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -843,9 +1039,8 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1158,13 +1353,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>104</v>
+        <v>121</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>105</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -1190,31 +1385,31 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>127</v>
+        <v>146</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>129</v>
+        <v>148</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>125</v>
+        <v>144</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>121</v>
+        <v>140</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>122</v>
+        <v>141</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -1240,31 +1435,31 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>130</v>
+        <v>149</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>125</v>
+        <v>144</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>121</v>
+        <v>140</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>122</v>
+        <v>141</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -1292,43 +1487,43 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>133</v>
+        <v>152</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>134</v>
+        <v>153</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>138</v>
+        <v>157</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>139</v>
+        <v>158</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>125</v>
+        <v>144</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>121</v>
+        <v>140</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>122</v>
+        <v>141</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -1338,71 +1533,15 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
-  <dimension ref="A1:CD81"/>
+  <dimension ref="A1:CC81"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="33.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15" bestFit="1" customWidth="1"/>
-    <col min="15" max="22" width="16" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="32.7109375" bestFit="1" customWidth="1"/>
-    <col min="29" max="32" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="28.7109375" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="27" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="39" max="45" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="25.5703125" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="18" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="26.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="55" max="59" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="27.85546875" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="68" max="69" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="26.7109375" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="21" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="8" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="81" width="7.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:82" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:81" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>191</v>
+        <v>223</v>
       </c>
       <c r="B1" t="s">
         <v>16</v>
@@ -1644,81 +1783,78 @@
       <c r="CC1" t="s">
         <v>95</v>
       </c>
-      <c r="CD1" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="2" spans="1:82" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:81" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:82" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:81" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:82" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:81" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:82" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:81" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:82" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:81" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:82" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:81" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:82" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:81" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:82" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:81" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:82" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:81" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:82" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:81" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:82" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:81" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:82" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:81" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:82" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:81" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:82" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:81" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:82" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:81" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -2055,7 +2191,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
@@ -2073,149 +2209,43 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>196</v>
+        <v>228</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>197</v>
+        <v>229</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>198</v>
+        <v>230</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>192</v>
+        <v>224</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>194</v>
+        <v>226</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>130</v>
+        <v>149</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>121</v>
+        <v>140</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>122</v>
+        <v>141</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D2" s="4"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D3" s="4"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D4" s="4"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D5" s="4"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D6" s="4"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D7" s="4"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D8" s="4"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D9" s="4"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D10" s="4"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D11" s="4"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D12" s="4"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D13" s="4"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D14" s="4"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D15" s="4"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D16" s="4"/>
-    </row>
-    <row r="17" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D17" s="4"/>
-    </row>
-    <row r="18" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D18" s="4"/>
-    </row>
-    <row r="19" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D19" s="4"/>
-    </row>
-    <row r="20" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D20" s="4"/>
-    </row>
-    <row r="21" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D21" s="4"/>
-    </row>
-    <row r="22" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D22" s="4"/>
-    </row>
-    <row r="23" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D23" s="4"/>
-    </row>
-    <row r="24" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D24" s="4"/>
-    </row>
-    <row r="25" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D25" s="4"/>
-    </row>
-    <row r="26" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D26" s="4"/>
-    </row>
-    <row r="27" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D27" s="4"/>
-    </row>
-    <row r="28" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D28" s="4"/>
-    </row>
-    <row r="29" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D29" s="4"/>
-    </row>
-    <row r="30" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D30" s="4"/>
-    </row>
-    <row r="31" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D31" s="4"/>
-    </row>
-    <row r="32" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D32" s="4"/>
-    </row>
-    <row r="33" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D33" s="4"/>
-    </row>
-    <row r="34" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D34" s="4"/>
-    </row>
-    <row r="35" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D35" s="4"/>
-    </row>
-    <row r="36" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D36" s="4"/>
-    </row>
-    <row r="37" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D37" s="4"/>
-    </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2241,40 +2271,40 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>200</v>
+        <v>232</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>199</v>
+        <v>231</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>201</v>
+        <v>233</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>193</v>
+        <v>225</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>195</v>
+        <v>227</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>194</v>
+        <v>226</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>130</v>
+        <v>149</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>121</v>
+        <v>140</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>122</v>
+        <v>141</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -2300,31 +2330,31 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>202</v>
+        <v>234</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>203</v>
+        <v>235</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>204</v>
+        <v>236</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>205</v>
+        <v>237</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>206</v>
+        <v>238</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>207</v>
+        <v>239</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>121</v>
+        <v>140</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>122</v>
+        <v>141</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -2349,28 +2379,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>202</v>
+        <v>234</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>203</v>
+        <v>235</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>204</v>
+        <v>236</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>208</v>
+        <v>240</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>207</v>
+        <v>239</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>121</v>
+        <v>140</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>122</v>
+        <v>141</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -2382,159 +2412,22 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE4E35F8-7819-4E55-92CB-94AF21738FD2}">
-  <dimension ref="A1:A41"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4"/>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4"/>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4"/>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4"/>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4"/>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4"/>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4"/>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4"/>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="4"/>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="4"/>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="4"/>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="4"/>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="4"/>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="4"/>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="4"/>
-    </row>
-    <row r="17" spans="1:1" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A17" s="7"/>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="4"/>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="4"/>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="4"/>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="4"/>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" s="4"/>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" s="4"/>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" s="4"/>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" s="4"/>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" s="4"/>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" s="4"/>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" s="4"/>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" s="4"/>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" s="4"/>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31" s="4"/>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" s="4"/>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" s="4"/>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" s="4"/>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" s="4"/>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" s="4"/>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37" s="4"/>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" s="4"/>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" s="4"/>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40" s="4"/>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A41" s="4"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D8A8D90-B9D8-4E8E-B8C5-B87B3EDD59F1}">
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:R1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="11.85546875" customWidth="1"/>
-    <col min="5" max="6" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.85546875" customWidth="1"/>
     <col min="15" max="15" width="22" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="23.7109375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="19" bestFit="1" customWidth="1"/>
@@ -2542,103 +2435,124 @@
     <col min="19" max="19" width="10.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>209</v>
+        <v>241</v>
       </c>
       <c r="B1" t="s">
-        <v>210</v>
+        <v>242</v>
       </c>
       <c r="C1" t="s">
-        <v>96</v>
+        <v>243</v>
       </c>
       <c r="D1" t="s">
-        <v>233</v>
+        <v>244</v>
       </c>
       <c r="E1" t="s">
-        <v>97</v>
+        <v>245</v>
       </c>
       <c r="F1" t="s">
-        <v>211</v>
+        <v>246</v>
       </c>
       <c r="G1" t="s">
-        <v>212</v>
+        <v>247</v>
       </c>
       <c r="H1" t="s">
-        <v>213</v>
+        <v>248</v>
       </c>
       <c r="I1" t="s">
-        <v>214</v>
+        <v>249</v>
       </c>
       <c r="J1" t="s">
-        <v>215</v>
+        <v>250</v>
       </c>
       <c r="K1" t="s">
-        <v>229</v>
+        <v>288</v>
       </c>
       <c r="L1" t="s">
-        <v>230</v>
+        <v>291</v>
       </c>
       <c r="M1" t="s">
-        <v>216</v>
+        <v>290</v>
       </c>
       <c r="N1" t="s">
-        <v>217</v>
+        <v>297</v>
       </c>
       <c r="O1" t="s">
-        <v>218</v>
+        <v>253</v>
       </c>
       <c r="P1" t="s">
-        <v>219</v>
+        <v>254</v>
       </c>
       <c r="Q1" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>224</v>
-      </c>
-      <c r="L2" s="6"/>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>225</v>
-      </c>
-      <c r="L3" s="6"/>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
-        <v>226</v>
-      </c>
-      <c r="L4" s="6"/>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>227</v>
-      </c>
-      <c r="L5" s="6"/>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>228</v>
-      </c>
-      <c r="L6" s="6"/>
+        <v>251</v>
+      </c>
+      <c r="R1" t="s">
+        <v>252</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22DCE508-4EF3-4CE2-915A-C48C27323B08}">
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>283</v>
+      </c>
+      <c r="B1" t="s">
+        <v>284</v>
+      </c>
+      <c r="C1" t="s">
+        <v>285</v>
+      </c>
+      <c r="D1" t="s">
+        <v>286</v>
+      </c>
+      <c r="E1" t="s">
+        <v>276</v>
+      </c>
+      <c r="F1" t="s">
+        <v>277</v>
+      </c>
+      <c r="G1" t="s">
+        <v>278</v>
+      </c>
+      <c r="H1" t="s">
+        <v>279</v>
+      </c>
+      <c r="I1" t="s">
+        <v>280</v>
+      </c>
+      <c r="J1" t="s">
+        <v>281</v>
+      </c>
+      <c r="K1" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D2" s="4"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D3" s="4"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D4" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -2647,64 +2561,32 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:M1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="23" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>2</v>
+        <v>123</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>3</v>
+        <v>124</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>4</v>
+        <v>125</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
     </row>
   </sheetData>
@@ -2714,752 +2596,942 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22DCE508-4EF3-4CE2-915A-C48C27323B08}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18FE2BAD-419E-4653-8809-5C67056F6E86}">
+  <dimension ref="A1:U5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.42578125" customWidth="1"/>
+    <col min="14" max="14" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.5703125" customWidth="1"/>
+    <col min="16" max="16" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="19.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>255</v>
+      </c>
+      <c r="B1" t="s">
+        <v>256</v>
+      </c>
+      <c r="C1" t="s">
+        <v>257</v>
+      </c>
+      <c r="D1" t="s">
+        <v>258</v>
+      </c>
+      <c r="E1" t="s">
+        <v>266</v>
+      </c>
+      <c r="F1" t="s">
+        <v>264</v>
+      </c>
+      <c r="G1" t="s">
+        <v>265</v>
+      </c>
+      <c r="H1" t="s">
+        <v>263</v>
+      </c>
+      <c r="I1" t="s">
+        <v>259</v>
+      </c>
+      <c r="J1" t="s">
+        <v>260</v>
+      </c>
+      <c r="K1" t="s">
+        <v>267</v>
+      </c>
+      <c r="L1" t="s">
+        <v>268</v>
+      </c>
+      <c r="M1" t="s">
+        <v>275</v>
+      </c>
+      <c r="N1" t="s">
+        <v>261</v>
+      </c>
+      <c r="O1" t="s">
+        <v>262</v>
+      </c>
+      <c r="P1" t="s">
+        <v>271</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>272</v>
+      </c>
+      <c r="R1" t="s">
+        <v>273</v>
+      </c>
+      <c r="S1" t="s">
+        <v>274</v>
+      </c>
+      <c r="T1" t="s">
+        <v>269</v>
+      </c>
+      <c r="U1" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5"/>
+      <c r="P2" s="5"/>
+      <c r="Q2" s="5"/>
+      <c r="S2" s="5"/>
+      <c r="T2" s="5"/>
+      <c r="U2" s="5"/>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="P3" s="5"/>
+      <c r="Q3" s="5"/>
+      <c r="S3" s="5"/>
+      <c r="T3" s="5"/>
+      <c r="U3" s="5"/>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="5"/>
+      <c r="P4" s="5"/>
+      <c r="Q4" s="5"/>
+      <c r="R4" s="5"/>
+      <c r="S4" s="5"/>
+      <c r="T4" s="5"/>
+      <c r="U4" s="5"/>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="5"/>
+      <c r="P5" s="5"/>
+      <c r="Q5" s="5"/>
+      <c r="S5" s="5"/>
+      <c r="T5" s="5"/>
+      <c r="U5" s="5"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18FE2BAD-419E-4653-8809-5C67056F6E86}">
-  <dimension ref="A1:II1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE4E35F8-7819-4E55-92CB-94AF21738FD2}">
+  <dimension ref="A1:C61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:243" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>220</v>
+        <v>295</v>
       </c>
       <c r="B1" t="s">
-        <v>221</v>
+        <v>287</v>
       </c>
       <c r="C1" t="s">
-        <v>222</v>
-      </c>
-      <c r="D1" s="8">
-        <v>0</v>
-      </c>
-      <c r="E1" s="8">
-        <v>4.1666666666666666E-3</v>
-      </c>
-      <c r="F1" s="8">
-        <v>8.3333333333333297E-3</v>
-      </c>
-      <c r="G1" s="8">
-        <v>1.2500000000000001E-2</v>
-      </c>
-      <c r="H1" s="8">
-        <v>1.6666666666666701E-2</v>
-      </c>
-      <c r="I1" s="8">
-        <v>2.0833333333333301E-2</v>
-      </c>
-      <c r="J1" s="8">
-        <v>2.5000000000000001E-2</v>
-      </c>
-      <c r="K1" s="8">
-        <v>2.9166666666666698E-2</v>
-      </c>
-      <c r="L1" s="8">
-        <v>3.3333333333333298E-2</v>
-      </c>
-      <c r="M1" s="8">
-        <v>3.7499999999999999E-2</v>
-      </c>
-      <c r="N1" s="8">
-        <v>4.1666666666666699E-2</v>
-      </c>
-      <c r="O1" s="8">
-        <v>4.5833333333333302E-2</v>
-      </c>
-      <c r="P1" s="8">
-        <v>0.05</v>
-      </c>
-      <c r="Q1" s="8">
-        <v>5.4166666666666703E-2</v>
-      </c>
-      <c r="R1" s="8">
-        <v>5.83333333333333E-2</v>
-      </c>
-      <c r="S1" s="8">
-        <v>6.25E-2</v>
-      </c>
-      <c r="T1" s="8">
-        <v>6.6666666666666693E-2</v>
-      </c>
-      <c r="U1" s="8">
-        <v>7.0833333333333304E-2</v>
-      </c>
-      <c r="V1" s="8">
-        <v>7.4999999999999997E-2</v>
-      </c>
-      <c r="W1" s="8">
-        <v>7.9166666666666705E-2</v>
-      </c>
-      <c r="X1" s="8">
-        <v>8.3333333333333301E-2</v>
-      </c>
-      <c r="Y1" s="8">
-        <v>8.7499999999999994E-2</v>
-      </c>
-      <c r="Z1" s="8">
-        <v>9.1666666666666702E-2</v>
-      </c>
-      <c r="AA1" s="8">
-        <v>9.5833333333333298E-2</v>
-      </c>
-      <c r="AB1" s="8">
-        <v>0.1</v>
-      </c>
-      <c r="AC1" s="8">
-        <v>0.104166666666667</v>
-      </c>
-      <c r="AD1" s="8">
-        <v>0.108333333333333</v>
-      </c>
-      <c r="AE1" s="8">
-        <v>0.1125</v>
-      </c>
-      <c r="AF1" s="8">
-        <v>0.116666666666667</v>
-      </c>
-      <c r="AG1" s="8">
-        <v>0.120833333333333</v>
-      </c>
-      <c r="AH1" s="8">
-        <v>0.125</v>
-      </c>
-      <c r="AI1" s="8">
-        <v>0.12916666666666701</v>
-      </c>
-      <c r="AJ1" s="8">
-        <v>0.133333333333333</v>
-      </c>
-      <c r="AK1" s="8">
-        <v>0.13750000000000001</v>
-      </c>
-      <c r="AL1" s="8">
-        <v>0.141666666666667</v>
-      </c>
-      <c r="AM1" s="8">
-        <v>0.14583333333333301</v>
-      </c>
-      <c r="AN1" s="8">
-        <v>0.15</v>
-      </c>
-      <c r="AO1" s="8">
-        <v>0.15416666666666701</v>
-      </c>
-      <c r="AP1" s="8">
-        <v>0.15833333333333299</v>
-      </c>
-      <c r="AQ1" s="8">
-        <v>0.16250000000000001</v>
-      </c>
-      <c r="AR1" s="8">
-        <v>0.16666666666666699</v>
-      </c>
-      <c r="AS1" s="8">
-        <v>0.170833333333333</v>
-      </c>
-      <c r="AT1" s="8">
-        <v>0.17499999999999999</v>
-      </c>
-      <c r="AU1" s="8">
-        <v>0.179166666666667</v>
-      </c>
-      <c r="AV1" s="8">
-        <v>0.18333333333333299</v>
-      </c>
-      <c r="AW1" s="8">
-        <v>0.1875</v>
-      </c>
-      <c r="AX1" s="8">
-        <v>0.19166666666666701</v>
-      </c>
-      <c r="AY1" s="8">
-        <v>0.195833333333333</v>
-      </c>
-      <c r="AZ1" s="8">
-        <v>0.2</v>
-      </c>
-      <c r="BA1" s="8">
-        <v>0.204166666666667</v>
-      </c>
-      <c r="BB1" s="8">
-        <v>0.20833333333333301</v>
-      </c>
-      <c r="BC1" s="8">
-        <v>0.21249999999999999</v>
-      </c>
-      <c r="BD1" s="8">
-        <v>0.21666666666666701</v>
-      </c>
-      <c r="BE1" s="8">
-        <v>0.22083333333333299</v>
-      </c>
-      <c r="BF1" s="8">
-        <v>0.22500000000000001</v>
-      </c>
-      <c r="BG1" s="8">
-        <v>0.22916666666666699</v>
-      </c>
-      <c r="BH1" s="8">
-        <v>0.233333333333333</v>
-      </c>
-      <c r="BI1" s="8">
-        <v>0.23749999999999999</v>
-      </c>
-      <c r="BJ1" s="8">
-        <v>0.241666666666667</v>
-      </c>
-      <c r="BK1" s="8">
-        <v>0.24583333333333299</v>
-      </c>
-      <c r="BL1" s="8">
-        <v>0.25</v>
-      </c>
-      <c r="BM1" s="8">
-        <v>0.25416666666666698</v>
-      </c>
-      <c r="BN1" s="8">
-        <v>0.25833333333333303</v>
-      </c>
-      <c r="BO1" s="8">
-        <v>0.26250000000000001</v>
-      </c>
-      <c r="BP1" s="8">
-        <v>0.266666666666667</v>
-      </c>
-      <c r="BQ1" s="8">
-        <v>0.27083333333333298</v>
-      </c>
-      <c r="BR1" s="8">
-        <v>0.27500000000000002</v>
-      </c>
-      <c r="BS1" s="8">
-        <v>0.27916666666666701</v>
-      </c>
-      <c r="BT1" s="8">
-        <v>0.28333333333333299</v>
-      </c>
-      <c r="BU1" s="8">
-        <v>0.28749999999999998</v>
-      </c>
-      <c r="BV1" s="8">
-        <v>0.29166666666666702</v>
-      </c>
-      <c r="BW1" s="8">
-        <v>0.295833333333333</v>
-      </c>
-      <c r="BX1" s="8">
-        <v>0.3</v>
-      </c>
-      <c r="BY1" s="8">
-        <v>0.30416666666666697</v>
-      </c>
-      <c r="BZ1" s="8">
-        <v>0.30833333333333302</v>
-      </c>
-      <c r="CA1" s="8">
-        <v>0.3125</v>
-      </c>
-      <c r="CB1" s="8">
-        <v>0.31666666666666698</v>
-      </c>
-      <c r="CC1" s="8">
-        <v>0.32083333333333303</v>
-      </c>
-      <c r="CD1" s="8">
-        <v>0.32500000000000001</v>
-      </c>
-      <c r="CE1" s="8">
-        <v>0.329166666666667</v>
-      </c>
-      <c r="CF1" s="8">
-        <v>0.33333333333333298</v>
-      </c>
-      <c r="CG1" s="8">
-        <v>0.33750000000000002</v>
-      </c>
-      <c r="CH1" s="8">
-        <v>0.34166666666666701</v>
-      </c>
-      <c r="CI1" s="8">
-        <v>0.34583333333333299</v>
-      </c>
-      <c r="CJ1" s="8">
-        <v>0.35</v>
-      </c>
-      <c r="CK1" s="8">
-        <v>0.35416666666666702</v>
-      </c>
-      <c r="CL1" s="8">
-        <v>0.358333333333333</v>
-      </c>
-      <c r="CM1" s="8">
-        <v>0.36249999999999999</v>
-      </c>
-      <c r="CN1" s="8">
-        <v>0.36666666666666697</v>
-      </c>
-      <c r="CO1" s="8">
-        <v>0.37083333333333302</v>
-      </c>
-      <c r="CP1" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="CQ1" s="8">
-        <v>0.37916666666666698</v>
-      </c>
-      <c r="CR1" s="8">
-        <v>0.38333333333333303</v>
-      </c>
-      <c r="CS1" s="8">
-        <v>0.38750000000000001</v>
-      </c>
-      <c r="CT1" s="8">
-        <v>0.391666666666667</v>
-      </c>
-      <c r="CU1" s="8">
-        <v>0.39583333333333298</v>
-      </c>
-      <c r="CV1" s="8">
-        <v>0.4</v>
-      </c>
-      <c r="CW1" s="8">
-        <v>0.40416666666666701</v>
-      </c>
-      <c r="CX1" s="8">
-        <v>0.40833333333333299</v>
-      </c>
-      <c r="CY1" s="8">
-        <v>0.41249999999999998</v>
-      </c>
-      <c r="CZ1" s="8">
-        <v>0.41666666666666702</v>
-      </c>
-      <c r="DA1" s="8">
-        <v>0.420833333333333</v>
-      </c>
-      <c r="DB1" s="8">
-        <v>0.42499999999999999</v>
-      </c>
-      <c r="DC1" s="8">
-        <v>0.42916666666666697</v>
-      </c>
-      <c r="DD1" s="8">
-        <v>0.43333333333333302</v>
-      </c>
-      <c r="DE1" s="8">
-        <v>0.4375</v>
-      </c>
-      <c r="DF1" s="8">
-        <v>0.44166666666666698</v>
-      </c>
-      <c r="DG1" s="8">
-        <v>0.44583333333333303</v>
-      </c>
-      <c r="DH1" s="8">
-        <v>0.45</v>
-      </c>
-      <c r="DI1" s="8">
-        <v>0.454166666666667</v>
-      </c>
-      <c r="DJ1" s="8">
-        <v>0.45833333333333298</v>
-      </c>
-      <c r="DK1" s="8">
-        <v>0.46250000000000002</v>
-      </c>
-      <c r="DL1" s="8">
-        <v>0.46666666666666701</v>
-      </c>
-      <c r="DM1" s="8">
-        <v>0.47083333333333299</v>
-      </c>
-      <c r="DN1" s="8">
-        <v>0.47499999999999998</v>
-      </c>
-      <c r="DO1" s="8">
-        <v>0.47916666666666702</v>
-      </c>
-      <c r="DP1" s="8">
-        <v>0.483333333333333</v>
-      </c>
-      <c r="DQ1" s="8">
-        <v>0.48749999999999999</v>
-      </c>
-      <c r="DR1" s="8">
-        <v>0.49166666666666697</v>
-      </c>
-      <c r="DS1" s="8">
-        <v>0.49583333333333302</v>
-      </c>
-      <c r="DT1" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="DU1" s="8">
-        <v>0.50416666666666698</v>
-      </c>
-      <c r="DV1" s="8">
-        <v>0.50833333333333297</v>
-      </c>
-      <c r="DW1" s="8">
-        <v>0.51249999999999996</v>
-      </c>
-      <c r="DX1" s="8">
-        <v>0.51666666666666705</v>
-      </c>
-      <c r="DY1" s="8">
-        <v>0.52083333333333304</v>
-      </c>
-      <c r="DZ1" s="8">
-        <v>0.52500000000000002</v>
-      </c>
-      <c r="EA1" s="8">
-        <v>0.52916666666666701</v>
-      </c>
-      <c r="EB1" s="8">
-        <v>0.53333333333333299</v>
-      </c>
-      <c r="EC1" s="8">
-        <v>0.53749999999999998</v>
-      </c>
-      <c r="ED1" s="8">
-        <v>0.54166666666666696</v>
-      </c>
-      <c r="EE1" s="8">
-        <v>0.54583333333333295</v>
-      </c>
-      <c r="EF1" s="8">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="EG1" s="8">
-        <v>0.55416666666666703</v>
-      </c>
-      <c r="EH1" s="8">
-        <v>0.55833333333333302</v>
-      </c>
-      <c r="EI1" s="8">
-        <v>0.5625</v>
-      </c>
-      <c r="EJ1" s="8">
-        <v>0.56666666666666698</v>
-      </c>
-      <c r="EK1" s="8">
-        <v>0.57083333333333297</v>
-      </c>
-      <c r="EL1" s="8">
-        <v>0.57499999999999996</v>
-      </c>
-      <c r="EM1" s="8">
-        <v>0.57916666666666705</v>
-      </c>
-      <c r="EN1" s="8">
-        <v>0.58333333333333304</v>
-      </c>
-      <c r="EO1" s="8">
-        <v>0.58750000000000002</v>
-      </c>
-      <c r="EP1" s="8">
-        <v>0.59166666666666701</v>
-      </c>
-      <c r="EQ1" s="8">
-        <v>0.59583333333333299</v>
-      </c>
-      <c r="ER1" s="8">
-        <v>0.6</v>
-      </c>
-      <c r="ES1" s="8">
-        <v>0.60416666666666696</v>
-      </c>
-      <c r="ET1" s="8">
-        <v>0.60833333333333295</v>
-      </c>
-      <c r="EU1" s="8">
-        <v>0.61250000000000004</v>
-      </c>
-      <c r="EV1" s="8">
-        <v>0.61666666666666703</v>
-      </c>
-      <c r="EW1" s="8">
-        <v>0.62083333333333302</v>
-      </c>
-      <c r="EX1" s="8">
-        <v>0.625</v>
-      </c>
-      <c r="EY1" s="8">
-        <v>0.62916666666666698</v>
-      </c>
-      <c r="EZ1" s="8">
-        <v>0.63333333333333297</v>
-      </c>
-      <c r="FA1" s="8">
-        <v>0.63749999999999996</v>
-      </c>
-      <c r="FB1" s="8">
-        <v>0.64166666666666705</v>
-      </c>
-      <c r="FC1" s="8">
-        <v>0.64583333333333304</v>
-      </c>
-      <c r="FD1" s="8">
-        <v>0.65</v>
-      </c>
-      <c r="FE1" s="8">
-        <v>0.65416666666666701</v>
-      </c>
-      <c r="FF1" s="8">
-        <v>0.65833333333333299</v>
-      </c>
-      <c r="FG1" s="8">
-        <v>0.66249999999999998</v>
-      </c>
-      <c r="FH1" s="8">
-        <v>0.66666666666666696</v>
-      </c>
-      <c r="FI1" s="8">
-        <v>0.67083333333333295</v>
-      </c>
-      <c r="FJ1" s="8">
-        <v>0.67500000000000004</v>
-      </c>
-      <c r="FK1" s="8">
-        <v>0.67916666666666703</v>
-      </c>
-      <c r="FL1" s="8">
-        <v>0.68333333333333302</v>
-      </c>
-      <c r="FM1" s="8">
-        <v>0.6875</v>
-      </c>
-      <c r="FN1" s="8">
-        <v>0.69166666666666698</v>
-      </c>
-      <c r="FO1" s="8">
-        <v>0.69583333333333297</v>
-      </c>
-      <c r="FP1" s="8">
-        <v>0.7</v>
-      </c>
-      <c r="FQ1" s="8">
-        <v>0.70416666666666705</v>
-      </c>
-      <c r="FR1" s="8">
-        <v>0.70833333333333304</v>
-      </c>
-      <c r="FS1" s="8">
-        <v>0.71250000000000002</v>
-      </c>
-      <c r="FT1" s="8">
-        <v>0.71666666666666701</v>
-      </c>
-      <c r="FU1" s="8">
-        <v>0.72083333333333299</v>
-      </c>
-      <c r="FV1" s="8">
-        <v>0.72499999999999998</v>
-      </c>
-      <c r="FW1" s="8">
-        <v>0.72916666666666696</v>
-      </c>
-      <c r="FX1" s="8">
-        <v>0.73333333333333295</v>
-      </c>
-      <c r="FY1" s="8">
-        <v>0.73750000000000004</v>
-      </c>
-      <c r="FZ1" s="8">
-        <v>0.74166666666666703</v>
-      </c>
-      <c r="GA1" s="8">
-        <v>0.74583333333333302</v>
-      </c>
-      <c r="GB1" s="8">
-        <v>0.75</v>
-      </c>
-      <c r="GC1" s="8">
-        <v>0.75416666666666698</v>
-      </c>
-      <c r="GD1" s="8">
-        <v>0.75833333333333297</v>
-      </c>
-      <c r="GE1" s="8">
-        <v>0.76249999999999996</v>
-      </c>
-      <c r="GF1" s="8">
-        <v>0.76666666666666705</v>
-      </c>
-      <c r="GG1" s="8">
-        <v>0.77083333333333304</v>
-      </c>
-      <c r="GH1" s="8">
-        <v>0.77500000000000002</v>
-      </c>
-      <c r="GI1" s="8">
-        <v>0.77916666666666701</v>
-      </c>
-      <c r="GJ1" s="8">
-        <v>0.78333333333333299</v>
-      </c>
-      <c r="GK1" s="8">
-        <v>0.78749999999999998</v>
-      </c>
-      <c r="GL1" s="8">
-        <v>0.79166666666666696</v>
-      </c>
-      <c r="GM1" s="8">
-        <v>0.79583333333333295</v>
-      </c>
-      <c r="GN1" s="8">
-        <v>0.8</v>
-      </c>
-      <c r="GO1" s="8">
-        <v>0.80416666666666703</v>
-      </c>
-      <c r="GP1" s="8">
-        <v>0.80833333333333302</v>
-      </c>
-      <c r="GQ1" s="8">
-        <v>0.8125</v>
-      </c>
-      <c r="GR1" s="8">
-        <v>0.81666666666666698</v>
-      </c>
-      <c r="GS1" s="8">
-        <v>0.82083333333333297</v>
-      </c>
-      <c r="GT1" s="8">
-        <v>0.82499999999999996</v>
-      </c>
-      <c r="GU1" s="8">
-        <v>0.82916666666666705</v>
-      </c>
-      <c r="GV1" s="8">
-        <v>0.83333333333333304</v>
-      </c>
-      <c r="GW1" s="8">
-        <v>0.83750000000000002</v>
-      </c>
-      <c r="GX1" s="8">
-        <v>0.84166666666666701</v>
-      </c>
-      <c r="GY1" s="8">
-        <v>0.84583333333333299</v>
-      </c>
-      <c r="GZ1" s="8">
-        <v>0.85</v>
-      </c>
-      <c r="HA1" s="8">
-        <v>0.85416666666666696</v>
-      </c>
-      <c r="HB1" s="8">
-        <v>0.85833333333333295</v>
-      </c>
-      <c r="HC1" s="8">
-        <v>0.86250000000000004</v>
-      </c>
-      <c r="HD1" s="8">
-        <v>0.86666666666666703</v>
-      </c>
-      <c r="HE1" s="8">
-        <v>0.87083333333333302</v>
-      </c>
-      <c r="HF1" s="8">
-        <v>0.875</v>
-      </c>
-      <c r="HG1" s="8">
-        <v>0.87916666666666698</v>
-      </c>
-      <c r="HH1" s="8">
-        <v>0.88333333333333297</v>
-      </c>
-      <c r="HI1" s="8">
-        <v>0.88749999999999996</v>
-      </c>
-      <c r="HJ1" s="8">
-        <v>0.89166666666666705</v>
-      </c>
-      <c r="HK1" s="8">
-        <v>0.89583333333333304</v>
-      </c>
-      <c r="HL1" s="8">
-        <v>0.9</v>
-      </c>
-      <c r="HM1" s="8">
-        <v>0.90416666666666701</v>
-      </c>
-      <c r="HN1" s="8">
-        <v>0.90833333333333299</v>
-      </c>
-      <c r="HO1" s="8">
-        <v>0.91249999999999998</v>
-      </c>
-      <c r="HP1" s="8">
-        <v>0.91666666666666696</v>
-      </c>
-      <c r="HQ1" s="8">
-        <v>0.92083333333333295</v>
-      </c>
-      <c r="HR1" s="8">
-        <v>0.92500000000000004</v>
-      </c>
-      <c r="HS1" s="8">
-        <v>0.92916666666666703</v>
-      </c>
-      <c r="HT1" s="8">
-        <v>0.93333333333333302</v>
-      </c>
-      <c r="HU1" s="8">
-        <v>0.9375</v>
-      </c>
-      <c r="HV1" s="8">
-        <v>0.94166666666666698</v>
-      </c>
-      <c r="HW1" s="8">
-        <v>0.94583333333333297</v>
-      </c>
-      <c r="HX1" s="8">
-        <v>0.95</v>
-      </c>
-      <c r="HY1" s="8">
-        <v>0.95416666666666705</v>
-      </c>
-      <c r="HZ1" s="8">
-        <v>0.95833333333333304</v>
-      </c>
-      <c r="IA1" s="8">
-        <v>0.96250000000000002</v>
-      </c>
-      <c r="IB1" s="8">
-        <v>0.96666666666666701</v>
-      </c>
-      <c r="IC1" s="8">
-        <v>0.97083333333333299</v>
-      </c>
-      <c r="ID1" s="8">
-        <v>0.97499999999999998</v>
-      </c>
-      <c r="IE1" s="8">
-        <v>0.97916666666666696</v>
-      </c>
-      <c r="IF1" s="8">
-        <v>0.98333333333333295</v>
-      </c>
-      <c r="IG1" s="8">
-        <v>0.98750000000000004</v>
-      </c>
-      <c r="IH1" s="8">
-        <v>0.99166666666666703</v>
-      </c>
-      <c r="II1" s="8">
-        <v>0.99583333333333302</v>
-      </c>
+        <v>294</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B2" s="4"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B3" s="7"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B4" s="4"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B5" s="4"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B6" s="4"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B7" s="4"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B8" s="4"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B9" s="4"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B10" s="4"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B11" s="4"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B12" s="4"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B13" s="4"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B14" s="4"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B15" s="7"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B16" s="4"/>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B17" s="4"/>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B18" s="4"/>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B19" s="4"/>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B20" s="4"/>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B21" s="4"/>
+    </row>
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B22" s="4"/>
+    </row>
+    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B23" s="4"/>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B24" s="4"/>
+    </row>
+    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B25" s="4"/>
+    </row>
+    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B26" s="4"/>
+    </row>
+    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B27" s="7"/>
+    </row>
+    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B28" s="4"/>
+    </row>
+    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B29" s="4"/>
+    </row>
+    <row r="30" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B30" s="4"/>
+    </row>
+    <row r="31" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B31" s="4"/>
+    </row>
+    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B32" s="4"/>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B33" s="4"/>
+    </row>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B34" s="4"/>
+    </row>
+    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B35" s="4"/>
+    </row>
+    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B36" s="4"/>
+    </row>
+    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B37" s="4"/>
+    </row>
+    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B38" s="4"/>
+    </row>
+    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B39" s="7"/>
+    </row>
+    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B40" s="4"/>
+    </row>
+    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B41" s="4"/>
+    </row>
+    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B42" s="4"/>
+    </row>
+    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B43" s="4"/>
+    </row>
+    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B44" s="4"/>
+    </row>
+    <row r="45" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B45" s="4"/>
+    </row>
+    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B46" s="4"/>
+    </row>
+    <row r="47" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B47" s="4"/>
+    </row>
+    <row r="48" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B48" s="4"/>
+    </row>
+    <row r="49" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B49" s="4"/>
+    </row>
+    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B50" s="4"/>
+    </row>
+    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B51" s="7"/>
+    </row>
+    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B52" s="4"/>
+    </row>
+    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B53" s="4"/>
+    </row>
+    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B54" s="4"/>
+    </row>
+    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B55" s="4"/>
+    </row>
+    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B56" s="4"/>
+    </row>
+    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B57" s="4"/>
+    </row>
+    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B58" s="4"/>
+    </row>
+    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B59" s="4"/>
+    </row>
+    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B60" s="4"/>
+    </row>
+    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B61" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDA296F8-8227-499C-B3D4-F942CBC18395}">
+  <dimension ref="A1:E181"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>296</v>
+      </c>
+      <c r="B1" t="s">
+        <v>289</v>
+      </c>
+      <c r="C1" t="s">
+        <v>292</v>
+      </c>
+      <c r="D1" t="s">
+        <v>292</v>
+      </c>
+      <c r="E1" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B2" s="4"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B3" s="4"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B4" s="4"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B5" s="4"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B6" s="4"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B7" s="4"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B8" s="4"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B9" s="4"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B10" s="4"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B11" s="4"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B12" s="4"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B13" s="4"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B14" s="4"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B15" s="4"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B16" s="4"/>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B17" s="4"/>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B18" s="4"/>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B19" s="4"/>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B20" s="4"/>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B21" s="4"/>
+    </row>
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B22" s="4"/>
+    </row>
+    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B23" s="4"/>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B24" s="4"/>
+    </row>
+    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B25" s="4"/>
+    </row>
+    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B26" s="4"/>
+    </row>
+    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B27" s="4"/>
+    </row>
+    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B28" s="4"/>
+    </row>
+    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B29" s="4"/>
+    </row>
+    <row r="30" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B30" s="4"/>
+    </row>
+    <row r="31" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B31" s="4"/>
+    </row>
+    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B32" s="4"/>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B33" s="4"/>
+    </row>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B34" s="4"/>
+    </row>
+    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B35" s="4"/>
+    </row>
+    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B36" s="4"/>
+    </row>
+    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B37" s="4"/>
+    </row>
+    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B38" s="4"/>
+    </row>
+    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B39" s="4"/>
+    </row>
+    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B40" s="4"/>
+    </row>
+    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B41" s="4"/>
+    </row>
+    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B42" s="4"/>
+    </row>
+    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B43" s="4"/>
+    </row>
+    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B44" s="4"/>
+    </row>
+    <row r="45" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B45" s="4"/>
+    </row>
+    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B46" s="4"/>
+    </row>
+    <row r="47" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B47" s="4"/>
+    </row>
+    <row r="48" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B48" s="4"/>
+    </row>
+    <row r="49" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B49" s="4"/>
+    </row>
+    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B50" s="4"/>
+    </row>
+    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B51" s="4"/>
+    </row>
+    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B52" s="4"/>
+    </row>
+    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B53" s="4"/>
+    </row>
+    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B54" s="4"/>
+    </row>
+    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B55" s="4"/>
+    </row>
+    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B56" s="4"/>
+    </row>
+    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B57" s="4"/>
+    </row>
+    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B58" s="4"/>
+    </row>
+    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B59" s="4"/>
+    </row>
+    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B60" s="4"/>
+    </row>
+    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B61" s="4"/>
+    </row>
+    <row r="62" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B62" s="4"/>
+    </row>
+    <row r="63" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B63" s="4"/>
+    </row>
+    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B64" s="4"/>
+    </row>
+    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B65" s="4"/>
+    </row>
+    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B66" s="4"/>
+    </row>
+    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B67" s="4"/>
+    </row>
+    <row r="68" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B68" s="4"/>
+    </row>
+    <row r="69" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B69" s="4"/>
+    </row>
+    <row r="70" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B70" s="4"/>
+    </row>
+    <row r="71" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B71" s="4"/>
+    </row>
+    <row r="72" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B72" s="4"/>
+    </row>
+    <row r="73" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B73" s="4"/>
+    </row>
+    <row r="74" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B74" s="4"/>
+    </row>
+    <row r="75" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B75" s="4"/>
+    </row>
+    <row r="76" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B76" s="4"/>
+    </row>
+    <row r="77" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B77" s="4"/>
+    </row>
+    <row r="78" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B78" s="4"/>
+    </row>
+    <row r="79" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B79" s="4"/>
+    </row>
+    <row r="80" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B80" s="4"/>
+    </row>
+    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B81" s="4"/>
+    </row>
+    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B82" s="4"/>
+    </row>
+    <row r="83" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B83" s="4"/>
+    </row>
+    <row r="84" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B84" s="4"/>
+    </row>
+    <row r="85" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B85" s="4"/>
+    </row>
+    <row r="86" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B86" s="4"/>
+    </row>
+    <row r="87" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B87" s="4"/>
+    </row>
+    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B88" s="4"/>
+    </row>
+    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B89" s="4"/>
+    </row>
+    <row r="90" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B90" s="4"/>
+    </row>
+    <row r="91" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B91" s="4"/>
+    </row>
+    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B92" s="4"/>
+    </row>
+    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B93" s="4"/>
+    </row>
+    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B94" s="4"/>
+    </row>
+    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B95" s="4"/>
+    </row>
+    <row r="96" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B96" s="4"/>
+    </row>
+    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B97" s="4"/>
+    </row>
+    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B98" s="4"/>
+    </row>
+    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B99" s="4"/>
+    </row>
+    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B100" s="4"/>
+    </row>
+    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B101" s="4"/>
+    </row>
+    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B102" s="4"/>
+    </row>
+    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B103" s="4"/>
+    </row>
+    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B104" s="4"/>
+    </row>
+    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B105" s="4"/>
+    </row>
+    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B106" s="4"/>
+    </row>
+    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B107" s="4"/>
+    </row>
+    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B108" s="4"/>
+    </row>
+    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B109" s="4"/>
+    </row>
+    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B110" s="4"/>
+    </row>
+    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B111" s="4"/>
+    </row>
+    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B112" s="4"/>
+    </row>
+    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B113" s="4"/>
+    </row>
+    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B114" s="4"/>
+    </row>
+    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B115" s="4"/>
+    </row>
+    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B116" s="4"/>
+    </row>
+    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B117" s="4"/>
+    </row>
+    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B118" s="4"/>
+    </row>
+    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B119" s="4"/>
+    </row>
+    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B120" s="4"/>
+    </row>
+    <row r="121" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B121" s="4"/>
+    </row>
+    <row r="122" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B122" s="4"/>
+    </row>
+    <row r="123" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B123" s="4"/>
+    </row>
+    <row r="124" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B124" s="4"/>
+    </row>
+    <row r="125" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B125" s="4"/>
+    </row>
+    <row r="126" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B126" s="4"/>
+    </row>
+    <row r="127" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B127" s="4"/>
+    </row>
+    <row r="128" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B128" s="4"/>
+    </row>
+    <row r="129" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B129" s="4"/>
+    </row>
+    <row r="130" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B130" s="4"/>
+    </row>
+    <row r="131" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B131" s="4"/>
+    </row>
+    <row r="132" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B132" s="4"/>
+    </row>
+    <row r="133" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B133" s="4"/>
+    </row>
+    <row r="134" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B134" s="4"/>
+    </row>
+    <row r="135" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B135" s="4"/>
+    </row>
+    <row r="136" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B136" s="4"/>
+    </row>
+    <row r="137" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B137" s="4"/>
+    </row>
+    <row r="138" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B138" s="4"/>
+    </row>
+    <row r="139" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B139" s="4"/>
+    </row>
+    <row r="140" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B140" s="4"/>
+    </row>
+    <row r="141" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B141" s="4"/>
+    </row>
+    <row r="142" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B142" s="4"/>
+    </row>
+    <row r="143" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B143" s="4"/>
+    </row>
+    <row r="144" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B144" s="4"/>
+    </row>
+    <row r="145" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B145" s="4"/>
+    </row>
+    <row r="146" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B146" s="4"/>
+    </row>
+    <row r="147" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B147" s="4"/>
+    </row>
+    <row r="148" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B148" s="4"/>
+    </row>
+    <row r="149" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B149" s="4"/>
+    </row>
+    <row r="150" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B150" s="4"/>
+    </row>
+    <row r="151" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B151" s="4"/>
+    </row>
+    <row r="152" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B152" s="4"/>
+    </row>
+    <row r="153" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B153" s="4"/>
+    </row>
+    <row r="154" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B154" s="4"/>
+    </row>
+    <row r="155" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B155" s="4"/>
+    </row>
+    <row r="156" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B156" s="4"/>
+    </row>
+    <row r="157" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B157" s="4"/>
+    </row>
+    <row r="158" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B158" s="4"/>
+    </row>
+    <row r="159" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B159" s="4"/>
+    </row>
+    <row r="160" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B160" s="4"/>
+    </row>
+    <row r="161" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B161" s="4"/>
+    </row>
+    <row r="162" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B162" s="4"/>
+    </row>
+    <row r="163" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B163" s="4"/>
+    </row>
+    <row r="164" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B164" s="4"/>
+    </row>
+    <row r="165" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B165" s="4"/>
+    </row>
+    <row r="166" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B166" s="4"/>
+    </row>
+    <row r="167" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B167" s="4"/>
+    </row>
+    <row r="168" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B168" s="4"/>
+    </row>
+    <row r="169" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B169" s="4"/>
+    </row>
+    <row r="170" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B170" s="4"/>
+    </row>
+    <row r="171" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B171" s="4"/>
+    </row>
+    <row r="172" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B172" s="4"/>
+    </row>
+    <row r="173" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B173" s="4"/>
+    </row>
+    <row r="174" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B174" s="4"/>
+    </row>
+    <row r="175" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B175" s="4"/>
+    </row>
+    <row r="176" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B176" s="4"/>
+    </row>
+    <row r="177" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B177" s="4"/>
+    </row>
+    <row r="178" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B178" s="4"/>
+    </row>
+    <row r="179" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B179" s="4"/>
+    </row>
+    <row r="180" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B180" s="4"/>
+    </row>
+    <row r="181" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B181" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3467,39 +3539,8 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.5703125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q82"/>
+  <dimension ref="A1:Q81"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
@@ -3530,7 +3571,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>140</v>
+        <v>159</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -3657,10 +3698,10 @@
       <c r="N28" s="5"/>
     </row>
     <row r="29" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="C29" s="2"/>
       <c r="N29" s="5"/>
     </row>
     <row r="30" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="C30" s="2"/>
       <c r="N30" s="5"/>
     </row>
     <row r="31" spans="3:14" x14ac:dyDescent="0.25">
@@ -3815,9 +3856,6 @@
     </row>
     <row r="81" spans="14:14" x14ac:dyDescent="0.25">
       <c r="N81" s="5"/>
-    </row>
-    <row r="82" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N82" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -3825,7 +3863,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E098E04-19A8-4E79-81CD-069FB2C95590}">
   <dimension ref="A1:BA30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3855,164 +3893,253 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:53" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="D1" t="s">
+        <v>160</v>
+      </c>
+      <c r="E1" t="s">
+        <v>161</v>
+      </c>
+      <c r="F1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G1" t="s">
+        <v>162</v>
+      </c>
+      <c r="H1" t="s">
+        <v>105</v>
+      </c>
+      <c r="I1" t="s">
+        <v>106</v>
+      </c>
+      <c r="J1" t="s">
+        <v>107</v>
+      </c>
+      <c r="K1" t="s">
+        <v>108</v>
+      </c>
+      <c r="L1" t="s">
+        <v>109</v>
+      </c>
+      <c r="M1" t="s">
+        <v>110</v>
+      </c>
+      <c r="N1" t="s">
+        <v>111</v>
+      </c>
+      <c r="O1" t="s">
+        <v>112</v>
+      </c>
+      <c r="P1" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>114</v>
+      </c>
+      <c r="R1" t="s">
+        <v>171</v>
+      </c>
+      <c r="S1" t="s">
+        <v>115</v>
+      </c>
+      <c r="T1" t="s">
+        <v>163</v>
+      </c>
+      <c r="U1" t="s">
+        <v>116</v>
+      </c>
+      <c r="V1" t="s">
+        <v>164</v>
+      </c>
+      <c r="W1" t="s">
+        <v>165</v>
+      </c>
+      <c r="X1" t="s">
+        <v>166</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>167</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>117</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>168</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>169</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>170</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>118</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>119</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="2" spans="1:53" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="V1" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="W1" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="AC1" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="AD1" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="AE1" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="AH1" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="AI1" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="AR1" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="AT1" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="AU1" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="AV1" s="1" t="s">
+      <c r="P2" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="AW1" s="1" t="s">
+      <c r="Q2" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="AX1" s="1" t="s">
+      <c r="R2" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="S2" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="AZ1" s="1" t="s">
+      <c r="T2" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="BA1" s="1" t="s">
+      <c r="U2" s="1" t="s">
         <v>190</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="X2" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="AB2" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="AC2" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="AD2" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="AE2" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="AF2" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AG2" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="AH2" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="AI2" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="AJ2" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="AK2" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="AL2" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="AM2" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="AN2" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="AO2" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="AP2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="AQ2" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="AR2" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="AS2" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="AT2" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="AU2" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="AV2" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="AW2" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="AX2" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="AY2" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="AZ2" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="BA2" s="1" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="30" spans="3:3" x14ac:dyDescent="0.25">
@@ -4024,7 +4151,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4044,28 +4171,95 @@
         <v>96</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>233</v>
+        <v>97</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4076,7 +4270,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="41.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21.42578125" bestFit="1" customWidth="1"/>
@@ -4091,22 +4285,22 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>133</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>115</v>
+        <v>134</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>116</v>
+        <v>135</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>118</v>
+        <v>137</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>2</v>
@@ -4118,13 +4312,13 @@
         <v>4</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>120</v>
+        <v>139</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>112</v>
+        <v>131</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -4145,13 +4339,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>121</v>
+        <v>140</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>122</v>
+        <v>141</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -4172,22 +4366,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>125</v>
+        <v>144</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>121</v>
+        <v>140</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>122</v>
+        <v>141</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>